<commit_message>
feat(F-NAR-016): TREE-DIF-042 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-042.xlsx
+++ b/stories/arbres/TREE-DIF-042.xlsx
@@ -1930,12 +1930,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La hanche porte le bidon, tout contre la robe. Il a trop de cacao ! C'est pour nos deux tasses. Victorino a les genoux plus hauts que Nina. Ses mains touchent déjà le bord du plan. Il est plus grand, c'est tout. On reste dans la cuisine ? Oui, papa.</t>
+          <t>La hanche porte le bidon, tout contre la robe. Il est tout froid ! Il va chauffer dans le lait. Victorino a les genoux plus hauts que Nina. Ses mains touchent déjà le bord du plan. Il est plus grand, c'est tout. On reste dans la cuisine ? Oui, papa.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La hanche porte le bidon, tout contre la robe. Il a trop de cacao ! C'est pour nos deux tasses. Victorino a les genoux plus hauts que Nina. Ses mains touchent déjà le bord du plan. Il est plus grand, c'est tout. On reste dans la cuisine ? Oui, papa.</t>
+          <t>La hanche porte le bidon, tout contre la robe. Il est tout froid ! Il va chauffer dans le lait. Victorino a les genoux plus hauts que Nina. Ses mains touchent déjà le bord du plan. Il est plus grand, c'est tout. On reste dans la cuisine ? Oui, papa.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2075,8 +2075,8 @@
       <c r="AW6" t="inlineStr">
         <is>
           <t>narrateur|La hanche porte le bidon, tout contre la robe.
-copain|Il a trop de cacao !
-enfant-f|C'est pour nos deux tasses.
+copain|Il est tout froid !
+enfant-f|Il va chauffer dans le lait.
 narrateur|Victorino a les genoux plus hauts que Nina.
 narrateur|Ses mains touchent déjà le bord du plan.
 maman|Il est plus grand, c'est tout.
@@ -2303,12 +2303,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Le bidon accroche une planche, trop haute. Le plan de travail sent le citron, trop haut. Moi je vois le fond du bol ! Victorino se hausse, trop vite. Ses doigts trouvent déjà le rebord froid. Un peu de poudre reste coincé dans le bois. Le bidon n'attendait pas ça. Tes bras n'arrivent pas encore. Lui voit le haut, toi le bois. On mélange comment, alors ? Vous faites comment, tous les deux ?</t>
+          <t>Nina pose le bidon sur le plan, trop haut. Le grand bol attend, trop loin pour Nina. Je ne vois plus le fond. Moi si, il est tout brun. Victorino se hausse, le menton au rebord. Un peu de poudre tombe, trop loin de ses yeux. Le bidon reste au-dessus d'elle, trop loin. Ses bras vont jusqu'au bol. Toi tu vois le bois, lui la poudre. On mélange comment, alors ? Vous faites comment, tous les deux ?</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Le bidon accroche une planche, trop haute. Le plan de travail sent le citron, trop haut. Moi je vois le fond du bol ! Victorino se hausse, trop vite. Ses doigts trouvent déjà le rebord froid. Un peu de poudre reste coincé dans le bois. Le bidon n'attendait pas ça. Tes bras n'arrivent pas encore. Lui voit le haut, toi le bois. On mélange comment, alors ? Vous faites comment, tous les deux ?</t>
+          <t>Nina pose le bidon sur le plan, trop haut. Le grand bol attend, trop loin pour Nina. Je ne vois plus le fond. Moi si, il est tout brun. Victorino se hausse, le menton au rebord. Un peu de poudre tombe, trop loin de ses yeux. Le bidon reste au-dessus d'elle, trop loin. Ses bras vont jusqu'au bol. Toi tu vois le bois, lui la poudre. On mélange comment, alors ? Vous faites comment, tous les deux ?</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2443,16 +2443,16 @@
       <c r="AV8" s="2" t="inlineStr"/>
       <c r="AW8" t="inlineStr">
         <is>
-          <t>narrateur|Le bidon accroche une planche, trop haute.
-narrateur|Le plan de travail sent le citron, trop haut.
-copain|Moi je vois le fond du bol !
-narrateur|Victorino se hausse, trop vite.
-narrateur|Ses doigts trouvent déjà le rebord froid.
-narrateur|Un peu de poudre reste coincé dans le bois.
-enfant-f|Le bidon n'attendait pas ça.
-maman|Tes bras n'arrivent pas encore.
-papa|Lui voit le haut, toi le bois.
-copain|On mélange comment, alors ?
+          <t>narrateur|Nina pose le bidon sur le plan, trop haut.
+narrateur|Le grand bol attend, trop loin pour Nina.
+enfant-f|Je ne vois plus le fond.
+copain|Moi si, il est tout brun.
+narrateur|Victorino se hausse, le menton au rebord.
+narrateur|Un peu de poudre tombe, trop loin de ses yeux.
+narrateur|Le bidon reste au-dessus d'elle, trop loin.
+maman|Ses bras vont jusqu'au bol.
+papa|Toi tu vois le bois, lui la poudre.
+enfant-f|On mélange comment, alors ?
 papa|Vous faites comment, tous les deux ?</t>
         </is>
       </c>
@@ -2676,12 +2676,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Tu mélanges, Victorino. Victorino lève le bol, assez haut. Doucement. Nina tend le bidon, bras tout courts. Ses doigts trouvent un rebord froid. Je tiens le bas ! Tes bras allaient assez loin. La poudre s'ouvre, à leur hauteur. Regarde, Nina. Il est à nous.</t>
+          <t>Tu mélanges, toi, tu vois le fond. Victorino tourne dans le bol, assez haut. Ça devient brun, tout doux. Nina tend le bidon, bras tout courts. Nina verse le lait, d'en bas, tout lent. Je tiens le pichet ! Tes bras allaient assez loin. La poudre s'ouvre, à leur hauteur. Goûte, Nina. Il est à nous.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Tu mélanges, Victorino. Victorino lève le bol, assez haut. Doucement. Nina tend le bidon, bras tout courts. Ses doigts trouvent un rebord froid. Je tiens le bas ! Tes bras allaient assez loin. La poudre s'ouvre, à leur hauteur. Regarde, Nina. Il est à nous.</t>
+          <t>Tu mélanges, toi, tu vois le fond. Victorino tourne dans le bol, assez haut. Ça devient brun, tout doux. Nina tend le bidon, bras tout courts. Nina verse le lait, d'en bas, tout lent. Je tiens le pichet ! Tes bras allaient assez loin. La poudre s'ouvre, à leur hauteur. Goûte, Nina. Il est à nous.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2816,15 +2816,15 @@
       <c r="AV10" s="2" t="inlineStr"/>
       <c r="AW10" t="inlineStr">
         <is>
-          <t>enfant-f|Tu mélanges, Victorino.
-narrateur|Victorino lève le bol, assez haut.
-copain|Doucement.
+          <t>enfant-f|Tu mélanges, toi, tu vois le fond.
+narrateur|Victorino tourne dans le bol, assez haut.
+copain|Ça devient brun, tout doux.
 narrateur|Nina tend le bidon, bras tout courts.
-narrateur|Ses doigts trouvent un rebord froid.
-enfant-f|Je tiens le bas !
+narrateur|Nina verse le lait, d'en bas, tout lent.
+enfant-f|Je tiens le pichet !
 papa|Tes bras allaient assez loin.
 narrateur|La poudre s'ouvre, à leur hauteur.
-copain|Regarde, Nina.
+copain|Goûte, Nina.
 enfant-f|Il est à nous.</t>
         </is>
       </c>
@@ -2852,12 +2852,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>À l'étagère, le cacao sent le citron. Tu tenais le bas, moi je mélangeais. Tes bras l'ont fait monter. Vous l'avez, enfin. Le bol dort sur le bois, au calme. Le bidon de cacao pèse encore sur le rebord. On reste un peu, Victorino. Un rai brun s'endort sur les carreaux. La buée redevient douce, dans l'air.</t>
+          <t>À l'étagère, le cacao sent le citron. Tu versais, moi je tournais. Tes bras ont vu le fond. Vous l'avez, enfin. Le bol dort sur le bois, au calme. Le bidon de cacao pèse encore sur le rebord. On reste un peu, Victorino. Un rai brun s'endort sur les carreaux. La buée redevient douce, dans l'air.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>À l'étagère, le cacao sent le citron. Tu tenais le bas, moi je mélangeais. Tes bras l'ont fait monter. Vous l'avez, enfin. Le bol dort sur le bois, au calme. Le bidon de cacao pèse encore sur le rebord. On reste un peu, Victorino. Un rai brun s'endort sur les carreaux. La buée redevient douce, dans l'air.</t>
+          <t>À l'étagère, le cacao sent le citron. Tu versais, moi je tournais. Tes bras ont vu le fond. Vous l'avez, enfin. Le bol dort sur le bois, au calme. Le bidon de cacao pèse encore sur le rebord. On reste un peu, Victorino. Un rai brun s'endort sur les carreaux. La buée redevient douce, dans l'air.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2993,8 +2993,8 @@
       <c r="AW11" t="inlineStr">
         <is>
           <t>narrateur|À l'étagère, le cacao sent le citron.
-copain|Tu tenais le bas, moi je mélangeais.
-enfant-f|Tes bras l'ont fait monter.
+copain|Tu versais, moi je tournais.
+enfant-f|Tes bras ont vu le fond.
 papa|Vous l'avez, enfin.
 maman|Le bol dort sur le bois, au calme.
 narrateur|Le bidon de cacao pèse encore sur le rebord.
@@ -3027,12 +3027,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Je monte, tout doux. Tiens le bois, Nina. Nina se hausse, plus petite que le bol. Moi je guide, tout près. Victorino tient le lait, au-dessus. La poudre glisse vers le fond. Il est à toi, un moment. Vous le partagez. Le bidon attend au bord, plein d'ombre.</t>
+          <t>Je monte, tout doux. Tiens le bois, Nina. Nina se hausse, le nez au bord du bol. Moi je verse le lait, tout près. Victorino tient le pichet, au-dessus. La poudre glisse vers le fond. Tu vois, maintenant. Vous le partagez. Le bidon attend au bord, plein d'ombre.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Je monte, tout doux. Tiens le bois, Nina. Nina se hausse, plus petite que le bol. Moi je guide, tout près. Victorino tient le lait, au-dessus. La poudre glisse vers le fond. Il est à toi, un moment. Vous le partagez. Le bidon attend au bord, plein d'ombre.</t>
+          <t>Je monte, tout doux. Tiens le bois, Nina. Nina se hausse, le nez au bord du bol. Moi je verse le lait, tout près. Victorino tient le pichet, au-dessus. La poudre glisse vers le fond. Tu vois, maintenant. Vous le partagez. Le bidon attend au bord, plein d'ombre.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -3169,11 +3169,11 @@
         <is>
           <t>enfant-f|Je monte, tout doux.
 papa|Tiens le bois, Nina.
-narrateur|Nina se hausse, plus petite que le bol.
-copain|Moi je guide, tout près.
-narrateur|Victorino tient le lait, au-dessus.
+narrateur|Nina se hausse, le nez au bord du bol.
+copain|Moi je verse le lait, tout près.
+narrateur|Victorino tient le pichet, au-dessus.
 narrateur|La poudre glisse vers le fond.
-copain|Il est à toi, un moment.
+copain|Tu vois, maintenant.
 maman|Vous le partagez.
 narrateur|Le bidon attend au bord, plein d'ombre.</t>
         </is>
@@ -3202,12 +3202,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Sur le tabouret, deux têtes se calment. Victorino, tu l'as vue glisser. Oui, tout près de tes mains. Toi en bas, lui au-dessus, ça tenait. Vos voix sont devenues toutes petites. Le bidon reste dans la paume de Nina. Je reste encore un peu. Une goutte reste collée au bol. L'évier sent encore le cacao.</t>
+          <t>Sur le tabouret, deux têtes se calment. J'ai vu le fond, moi aussi. Oui, tu étais assez haute. Toi en bas, lui au-dessus, ça tenait. Vos voix sont devenues toutes petites. Le bidon reste dans la paume de Nina. Je reste encore un peu. Une goutte reste collée au bol. L'évier sent encore le cacao.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Sur le tabouret, deux têtes se calment. Victorino, tu l'as vue glisser. Oui, tout près de tes mains. Toi en bas, lui au-dessus, ça tenait. Vos voix sont devenues toutes petites. Le bidon reste dans la paume de Nina. Je reste encore un peu. Une goutte reste collée au bol. L'évier sent encore le cacao.</t>
+          <t>Sur le tabouret, deux têtes se calment. J'ai vu le fond, moi aussi. Oui, tu étais assez haute. Toi en bas, lui au-dessus, ça tenait. Vos voix sont devenues toutes petites. Le bidon reste dans la paume de Nina. Je reste encore un peu. Une goutte reste collée au bol. L'évier sent encore le cacao.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -3343,8 +3343,8 @@
       <c r="AW13" t="inlineStr">
         <is>
           <t>narrateur|Sur le tabouret, deux têtes se calment.
-enfant-f|Victorino, tu l'as vue glisser.
-copain|Oui, tout près de tes mains.
+enfant-f|J'ai vu le fond, moi aussi.
+copain|Oui, tu étais assez haute.
 papa|Toi en bas, lui au-dessus, ça tenait.
 maman|Vos voix sont devenues toutes petites.
 narrateur|Le bidon reste dans la paume de Nina.
@@ -3377,12 +3377,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>On tire un peu. Moi aussi, je tire. Victorino lève un torchon, tout haut. Nina glisse le bol, pendant l'ouverture. Le bidon pince le torchon, tout doux. Il est venu vers vous. On l'a repris. Il fume encore. Vos cheveux sentent le linge chaud.</t>
+          <t>On tire le bol, tout doux. Moi aussi, je tire. Victorino enroule un torchon, tout haut. Nina tire l'autre bout, plus bas. Le bidon glisse avec le torchon, tout doux. Le bol est venu vers vous. On le tient. Il fume encore. Vos cheveux sentent le linge chaud.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>On tire un peu. Moi aussi, je tire. Victorino lève un torchon, tout haut. Nina glisse le bol, pendant l'ouverture. Le bidon pince le torchon, tout doux. Il est venu vers vous. On l'a repris. Il fume encore. Vos cheveux sentent le linge chaud.</t>
+          <t>On tire le bol, tout doux. Moi aussi, je tire. Victorino enroule un torchon, tout haut. Nina tire l'autre bout, plus bas. Le bidon glisse avec le torchon, tout doux. Le bol est venu vers vous. On le tient. Il fume encore. Vos cheveux sentent le linge chaud.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -3517,13 +3517,13 @@
       <c r="AV14" s="2" t="inlineStr"/>
       <c r="AW14" t="inlineStr">
         <is>
-          <t>enfant-f|On tire un peu.
+          <t>enfant-f|On tire le bol, tout doux.
 copain|Moi aussi, je tire.
-narrateur|Victorino lève un torchon, tout haut.
-narrateur|Nina glisse le bol, pendant l'ouverture.
-narrateur|Le bidon pince le torchon, tout doux.
-papa|Il est venu vers vous.
-copain|On l'a repris.
+narrateur|Victorino enroule un torchon, tout haut.
+narrateur|Nina tire l'autre bout, plus bas.
+narrateur|Le bidon glisse avec le torchon, tout doux.
+papa|Le bol est venu vers vous.
+copain|On le tient.
 enfant-f|Il fume encore.
 maman|Vos cheveux sentent le linge chaud.</t>
         </is>
@@ -3552,12 +3552,12 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Le torchon redescend, tout doux. Il est tombé vers nous. On a tiré, tous les deux. Il n'était plus trop coincé. La poudre froisse encore, dans l'air. Le bidon de cacao retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des bols. Le radiateur se tait, au fond.</t>
+          <t>Le torchon redescend, tout doux. Le bol est venu vers nous. On a tiré, tous les deux. Il n'était plus trop haut. La poudre danse encore, dans l'air. Le bidon de cacao retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des bols. Le radiateur se tait, au fond.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Le torchon redescend, tout doux. Il est tombé vers nous. On a tiré, tous les deux. Il n'était plus trop coincé. La poudre froisse encore, dans l'air. Le bidon de cacao retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des bols. Le radiateur se tait, au fond.</t>
+          <t>Le torchon redescend, tout doux. Le bol est venu vers nous. On a tiré, tous les deux. Il n'était plus trop haut. La poudre danse encore, dans l'air. Le bidon de cacao retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des bols. Le radiateur se tait, au fond.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -3693,10 +3693,10 @@
       <c r="AW15" t="inlineStr">
         <is>
           <t>narrateur|Le torchon redescend, tout doux.
-copain|Il est tombé vers nous.
+copain|Le bol est venu vers nous.
 enfant-f|On a tiré, tous les deux.
-maman|Il n'était plus trop coincé.
-papa|La poudre froisse encore, dans l'air.
+maman|Il n'était plus trop haut.
+papa|La poudre danse encore, dans l'air.
 narrateur|Le bidon de cacao retombe, tout léger.
 enfant-f|On souffle dessus, tout calme.
 narrateur|Un rayon veille près des bols.
@@ -3727,12 +3727,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Le bidon se colle à la porte, trop haute. Le lait est à nous, Victorino. Je vois le beurre, tout haut ! La poignée reste trop loin pour Nina. Le cacao reste trop bas, sous la poignée. Un peu d'air froid lève, puis retombe. Ses bras vont jusqu'à la poignée. Toi tu vois le bac, lui le beurre. On peut jouer avec lui ? Vous trouvez, tous les deux ?</t>
+          <t>Nina tape le bidon contre la porte, toc. Le lait est dedans, Victorino. Je vois déjà le beurre, tout haut ! La poignée reste trop loin pour Nina. Le cacao reste trop bas, sous la poignée. Un souffle froid lève, puis retombe. Ses bras vont jusqu'à la poignée. Toi tu vois le bac, lui le beurre. On ouvre comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Le bidon se colle à la porte, trop haute. Le lait est à nous, Victorino. Je vois le beurre, tout haut ! La poignée reste trop loin pour Nina. Le cacao reste trop bas, sous la poignée. Un peu d'air froid lève, puis retombe. Ses bras vont jusqu'à la poignée. Toi tu vois le bac, lui le beurre. On peut jouer avec lui ? Vous trouvez, tous les deux ?</t>
+          <t>Nina tape le bidon contre la porte, toc. Le lait est dedans, Victorino. Je vois déjà le beurre, tout haut ! La poignée reste trop loin pour Nina. Le cacao reste trop bas, sous la poignée. Un souffle froid lève, puis retombe. Ses bras vont jusqu'à la poignée. Toi tu vois le bac, lui le beurre. On ouvre comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -3867,15 +3867,15 @@
       <c r="AV16" s="2" t="inlineStr"/>
       <c r="AW16" t="inlineStr">
         <is>
-          <t>narrateur|Le bidon se colle à la porte, trop haute.
-enfant-f|Le lait est à nous, Victorino.
-copain|Je vois le beurre, tout haut !
+          <t>narrateur|Nina tape le bidon contre la porte, toc.
+enfant-f|Le lait est dedans, Victorino.
+copain|Je vois déjà le beurre, tout haut !
 narrateur|La poignée reste trop loin pour Nina.
 narrateur|Le cacao reste trop bas, sous la poignée.
-narrateur|Un peu d'air froid lève, puis retombe.
+narrateur|Un souffle froid lève, puis retombe.
 maman|Ses bras vont jusqu'à la poignée.
 papa|Toi tu vois le bac, lui le beurre.
-enfant-f|On peut jouer avec lui ?
+enfant-f|On ouvre comment, alors ?
 papa|Vous trouvez, tous les deux ?</t>
         </is>
       </c>
@@ -4099,12 +4099,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Je me hausse encore. Je tiens les tasses, d'en bas. Les doigts de Victorino touchent la poignée. Elle bouge ! Le lait penche, puis avance. Victorino pose le bidon contre la porte. Tes doigts allaient assez loin. Nina tenait bien le bas. Il est à nous.</t>
+          <t>Je me hausse encore. Je tiens les tasses, d'en bas. Les doigts de Victorino touchent la poignée. Elle bouge ! La bouteille de lait penche, puis avance. Victorino pose le bidon contre la porte. Tes doigts allaient assez loin. Nina tenait bien le bas. Le lait est à nous.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Je me hausse encore. Je tiens les tasses, d'en bas. Les doigts de Victorino touchent la poignée. Elle bouge ! Le lait penche, puis avance. Victorino pose le bidon contre la porte. Tes doigts allaient assez loin. Nina tenait bien le bas. Il est à nous.</t>
+          <t>Je me hausse encore. Je tiens les tasses, d'en bas. Les doigts de Victorino touchent la poignée. Elle bouge ! La bouteille de lait penche, puis avance. Victorino pose le bidon contre la porte. Tes doigts allaient assez loin. Nina tenait bien le bas. Le lait est à nous.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -4243,11 +4243,11 @@
 enfant-f|Je tiens les tasses, d'en bas.
 narrateur|Les doigts de Victorino touchent la poignée.
 copain|Elle bouge !
-narrateur|Le lait penche, puis avance.
+narrateur|La bouteille de lait penche, puis avance.
 narrateur|Victorino pose le bidon contre la porte.
 papa|Tes doigts allaient assez loin.
 maman|Nina tenait bien le bas.
-copain|Il est à nous.</t>
+copain|Le lait est à nous.</t>
         </is>
       </c>
     </row>
@@ -4274,12 +4274,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Au frigo, le cacao sent le lait. Tu l'as fait pencher pour moi. Tu tenais le bas. Le verre sent encore le matin. Le cacao est à vous, maintenant. Le bidon de cacao garde un brin de froid. Nina le verse contre la tasse petite. Un rai traverse la vapeur, tout chaud. Le loquet redevient calme, tout seul.</t>
+          <t>Au frigo, le cacao sent le lait. Tu as ouvert, tout haut. Tu tenais les tasses. Le verre sent encore le matin. Le cacao est à vous, maintenant. Le bidon de cacao garde un brin de froid. Nina verse dans la tasse petite. Un rai traverse la vapeur, tout chaud. Le loquet redevient calme, tout seul.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Au frigo, le cacao sent le lait. Tu l'as fait pencher pour moi. Tu tenais le bas. Le verre sent encore le matin. Le cacao est à vous, maintenant. Le bidon de cacao garde un brin de froid. Nina le verse contre la tasse petite. Un rai traverse la vapeur, tout chaud. Le loquet redevient calme, tout seul.</t>
+          <t>Au frigo, le cacao sent le lait. Tu as ouvert, tout haut. Tu tenais les tasses. Le verre sent encore le matin. Le cacao est à vous, maintenant. Le bidon de cacao garde un brin de froid. Nina verse dans la tasse petite. Un rai traverse la vapeur, tout chaud. Le loquet redevient calme, tout seul.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -4415,12 +4415,12 @@
       <c r="AW19" t="inlineStr">
         <is>
           <t>narrateur|Au frigo, le cacao sent le lait.
-enfant-f|Tu l'as fait pencher pour moi.
-copain|Tu tenais le bas.
+enfant-f|Tu as ouvert, tout haut.
+copain|Tu tenais les tasses.
 maman|Le verre sent encore le matin.
 papa|Le cacao est à vous, maintenant.
 narrateur|Le bidon de cacao garde un brin de froid.
-narrateur|Nina le verse contre la tasse petite.
+narrateur|Nina verse dans la tasse petite.
 narrateur|Un rai traverse la vapeur, tout chaud.
 narrateur|Le loquet redevient calme, tout seul.</t>
         </is>
@@ -4449,12 +4449,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>J'ouvre le bac du bas ? Oui, tout doux. Nina pose le bidon près du bac. Papa tient la porte, tout ferme. Nina tire le bac, Victorino veille. Le lait est là ! Je le sens. Vous avez regardé ensemble. Le bac est resté doux.</t>
+          <t>J'ouvre le bac du bas ? Oui, tout doux. Nina pose le bidon près du bac. Papa tient la porte, tout ferme. Nina tire le bac, Victorino veille. Le lait est là ! Il est tout froid. Vous avez regardé ensemble. Le bac est resté doux.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>J'ouvre le bac du bas ? Oui, tout doux. Nina pose le bidon près du bac. Papa tient la porte, tout ferme. Nina tire le bac, Victorino veille. Le lait est là ! Je le sens. Vous avez regardé ensemble. Le bac est resté doux.</t>
+          <t>J'ouvre le bac du bas ? Oui, tout doux. Nina pose le bidon près du bac. Papa tient la porte, tout ferme. Nina tire le bac, Victorino veille. Le lait est là ! Il est tout froid. Vous avez regardé ensemble. Le bac est resté doux.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -4595,7 +4595,7 @@
 narrateur|Papa tient la porte, tout ferme.
 narrateur|Nina tire le bac, Victorino veille.
 enfant-f|Le lait est là !
-copain|Je le sens.
+copain|Il est tout froid.
 maman|Vous avez regardé ensemble.
 papa|Le bac est resté doux.</t>
         </is>
@@ -4624,12 +4624,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Près du bac, deux paires de pieds se touchent. Tu l'as posé, d'en bas. Tes bras l'ont fait descendre. Chacun a fait sa part, à sa hauteur. Le bois du bac sèche déjà. Le bidon pose une ombre au bac. Il fume trop, Nina. C'est pour ça. La porte garde le froid, tout proche.</t>
+          <t>Près du bac, deux paires de pieds se touchent. Tu l'as trouvé, d'en bas. Tes yeux gardaient la porte. Chacun a fait sa part, à sa hauteur. Le bois du bac sèche déjà. Le bidon pose une ombre au bac. Il fume trop, Nina. C'est pour ça. La porte garde le froid, tout proche.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Près du bac, deux paires de pieds se touchent. Tu l'as posé, d'en bas. Tes bras l'ont fait descendre. Chacun a fait sa part, à sa hauteur. Le bois du bac sèche déjà. Le bidon pose une ombre au bac. Il fume trop, Nina. C'est pour ça. La porte garde le froid, tout proche.</t>
+          <t>Près du bac, deux paires de pieds se touchent. Tu l'as trouvé, d'en bas. Tes yeux gardaient la porte. Chacun a fait sa part, à sa hauteur. Le bois du bac sèche déjà. Le bidon pose une ombre au bac. Il fume trop, Nina. C'est pour ça. La porte garde le froid, tout proche.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -4765,8 +4765,8 @@
       <c r="AW21" t="inlineStr">
         <is>
           <t>narrateur|Près du bac, deux paires de pieds se touchent.
-copain|Tu l'as posé, d'en bas.
-enfant-f|Tes bras l'ont fait descendre.
+copain|Tu l'as trouvé, d'en bas.
+enfant-f|Tes yeux gardaient la porte.
 papa|Chacun a fait sa part, à sa hauteur.
 maman|Le bois du bac sèche déjà.
 narrateur|Le bidon pose une ombre au bac.
@@ -4799,12 +4799,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Reste en haut, Victorino. Je tends, d'ici. Victorino tend le bidon, bras tout longs. Victorino fait basculer le loquet, tout doux. Le tabouret prend Nina, puis lui. Je le tiens ! Chacun a fait sa part. Il sent le froid. Vos bras n'avaient pas la même longueur.</t>
+          <t>Reste en haut, Victorino. Je tends, d'ici. Victorino tend le bidon, bras tout longs. Victorino fait basculer le loquet, tout doux. Le tabouret prend Nina, puis lui. Je tiens la bouteille ! Chacun a fait sa part. Elle sent le froid. Vos bras n'avaient pas la même longueur.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Reste en haut, Victorino. Je tends, d'ici. Victorino tend le bidon, bras tout longs. Victorino fait basculer le loquet, tout doux. Le tabouret prend Nina, puis lui. Je le tiens ! Chacun a fait sa part. Il sent le froid. Vos bras n'avaient pas la même longueur.</t>
+          <t>Reste en haut, Victorino. Je tends, d'ici. Victorino tend le bidon, bras tout longs. Victorino fait basculer le loquet, tout doux. Le tabouret prend Nina, puis lui. Je tiens la bouteille ! Chacun a fait sa part. Elle sent le froid. Vos bras n'avaient pas la même longueur.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -4944,9 +4944,9 @@
 narrateur|Victorino tend le bidon, bras tout longs.
 narrateur|Victorino fait basculer le loquet, tout doux.
 narrateur|Le tabouret prend Nina, puis lui.
-enfant-f|Je le tiens !
+enfant-f|Je tiens la bouteille !
 papa|Chacun a fait sa part.
-copain|Il sent le froid.
+copain|Elle sent le froid.
 maman|Vos bras n'avaient pas la même longueur.</t>
         </is>
       </c>
@@ -4974,12 +4974,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Un peu de buée reste au frigo. On a tiré ensemble. Sans trop monter. Le tabouret est resté à sa place. Vos mains sentent encore le lait. Nina pose le bidon au rebord. Tu l'as eu, enfin. Il est à nous. La vapeur tremble un peu, puis s'endort.</t>
+          <t>Un peu de buée reste au frigo. On a ouvert ensemble. Sans trop monter. Le tabouret est resté à sa place. Vos mains sentent encore le lait. Nina pose le bidon au rebord. Tu l'as eu, enfin. Il est à nous. La vapeur tremble un peu, puis s'endort.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Un peu de buée reste au frigo. On a tiré ensemble. Sans trop monter. Le tabouret est resté à sa place. Vos mains sentent encore le lait. Nina pose le bidon au rebord. Tu l'as eu, enfin. Il est à nous. La vapeur tremble un peu, puis s'endort.</t>
+          <t>Un peu de buée reste au frigo. On a ouvert ensemble. Sans trop monter. Le tabouret est resté à sa place. Vos mains sentent encore le lait. Nina pose le bidon au rebord. Tu l'as eu, enfin. Il est à nous. La vapeur tremble un peu, puis s'endort.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -5115,7 +5115,7 @@
       <c r="AW23" t="inlineStr">
         <is>
           <t>narrateur|Un peu de buée reste au frigo.
-enfant-f|On a tiré ensemble.
+enfant-f|On a ouvert ensemble.
 copain|Sans trop monter.
 papa|Le tabouret est resté à sa place.
 maman|Vos mains sentent encore le lait.
@@ -5149,12 +5149,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Le bidon rampe sous la table, trop bas. Ici, ça sent le bois, Victorino. Je me glisse, trop large ! Ses épaules butent contre le bois de la table. Le cacao prend la poussière des carreaux. Le bidon attend au bord, un peu seul. Il a les épaules trop larges, c'est tout. Toi tu passes, lui pas encore. On joue comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>Nina glisse le bidon sous la table, tout bas. On goûte ici, comme une grotte. J'entre, trop large ! Ses épaules butent contre le bois de la table. Le cacao prend une miette, sur les carreaux. Le bidon attend au bord, un peu seul. Il a les épaules trop larges, c'est tout. Toi tu passes, lui pas encore. On goûte comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Le bidon rampe sous la table, trop bas. Ici, ça sent le bois, Victorino. Je me glisse, trop large ! Ses épaules butent contre le bois de la table. Le cacao prend la poussière des carreaux. Le bidon attend au bord, un peu seul. Il a les épaules trop larges, c'est tout. Toi tu passes, lui pas encore. On joue comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>Nina glisse le bidon sous la table, tout bas. On goûte ici, comme une grotte. J'entre, trop large ! Ses épaules butent contre le bois de la table. Le cacao prend une miette, sur les carreaux. Le bidon attend au bord, un peu seul. Il a les épaules trop larges, c'est tout. Toi tu passes, lui pas encore. On goûte comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -5289,15 +5289,15 @@
       <c r="AV24" s="2" t="inlineStr"/>
       <c r="AW24" t="inlineStr">
         <is>
-          <t>narrateur|Le bidon rampe sous la table, trop bas.
-enfant-f|Ici, ça sent le bois, Victorino.
-copain|Je me glisse, trop large !
+          <t>narrateur|Nina glisse le bidon sous la table, tout bas.
+enfant-f|On goûte ici, comme une grotte.
+copain|J'entre, trop large !
 narrateur|Ses épaules butent contre le bois de la table.
-narrateur|Le cacao prend la poussière des carreaux.
+narrateur|Le cacao prend une miette, sur les carreaux.
 narrateur|Le bidon attend au bord, un peu seul.
 maman|Il a les épaules trop larges, c'est tout.
 papa|Toi tu passes, lui pas encore.
-copain|On joue comment, alors ?
+copain|On goûte comment, alors ?
 papa|Vous trouvez, tous les deux ?</t>
         </is>
       </c>
@@ -5521,12 +5521,12 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Je passe, Victorino. Nina rampe, tout petite, sous la table. Doucement. Nina pousse le bidon sous la table. Ses doigts trouvent une cuillère perdue. Je la tiens ! Tes épaules étaient assez petites. Une grotte de lumière s'ouvre, à eux. Regarde, Nina. Elle est à nous.</t>
+          <t>Je passe, toi tu restes. Nina rampe, tout petite, sous la table. Je fouette ici, dehors. Nina pousse le bidon sous la table. Ses doigts trouvent la petite tasse. Je la tiens ! Tes épaules étaient assez petites. Une grotte de vapeur s'ouvre, à eux. Je te verse, d'ici. Elle est à nous.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Je passe, Victorino. Nina rampe, tout petite, sous la table. Doucement. Nina pousse le bidon sous la table. Ses doigts trouvent une cuillère perdue. Je la tiens ! Tes épaules étaient assez petites. Une grotte de lumière s'ouvre, à eux. Regarde, Nina. Elle est à nous.</t>
+          <t>Je passe, toi tu restes. Nina rampe, tout petite, sous la table. Je fouette ici, dehors. Nina pousse le bidon sous la table. Ses doigts trouvent la petite tasse. Je la tiens ! Tes épaules étaient assez petites. Une grotte de vapeur s'ouvre, à eux. Je te verse, d'ici. Elle est à nous.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -5661,15 +5661,15 @@
       <c r="AV26" s="2" t="inlineStr"/>
       <c r="AW26" t="inlineStr">
         <is>
-          <t>enfant-f|Je passe, Victorino.
+          <t>enfant-f|Je passe, toi tu restes.
 narrateur|Nina rampe, tout petite, sous la table.
-copain|Doucement.
+copain|Je fouette ici, dehors.
 narrateur|Nina pousse le bidon sous la table.
-narrateur|Ses doigts trouvent une cuillère perdue.
+narrateur|Ses doigts trouvent la petite tasse.
 enfant-f|Je la tiens !
 papa|Tes épaules étaient assez petites.
-narrateur|Une grotte de lumière s'ouvre, à eux.
-copain|Regarde, Nina.
+narrateur|Une grotte de vapeur s'ouvre, à eux.
+copain|Je te verse, d'ici.
 enfant-f|Elle est à nous.</t>
         </is>
       </c>
@@ -5697,12 +5697,12 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Sous la table, la grotte sent le bois. Tu es passée, moi je gardais. Tes épaules l'ont laissé ouvert. Vous l'avez, enfin. La cuillère dort sur le bord, au calme. Le bidon de cacao couvre encore leurs genoux. On reste un peu, Victorino. Un rai brun s'endort sous le bois. La poussière redevient douce, autour.</t>
+          <t>Sous la table, la grotte sent le bois. Tu es passée, moi je fouettais. Tes épaules l'ont laissé ouvert. Vous l'avez, enfin. La petite tasse dort sur le bord, au calme. Le bidon de cacao couvre encore leurs genoux. On reste un peu, Victorino. Un rai brun s'endort sous le bois. La miette redevient douce, autour.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Sous la table, la grotte sent le bois. Tu es passée, moi je gardais. Tes épaules l'ont laissé ouvert. Vous l'avez, enfin. La cuillère dort sur le bord, au calme. Le bidon de cacao couvre encore leurs genoux. On reste un peu, Victorino. Un rai brun s'endort sous le bois. La poussière redevient douce, autour.</t>
+          <t>Sous la table, la grotte sent le bois. Tu es passée, moi je fouettais. Tes épaules l'ont laissé ouvert. Vous l'avez, enfin. La petite tasse dort sur le bord, au calme. Le bidon de cacao couvre encore leurs genoux. On reste un peu, Victorino. Un rai brun s'endort sous le bois. La miette redevient douce, autour.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -5838,14 +5838,14 @@
       <c r="AW27" t="inlineStr">
         <is>
           <t>narrateur|Sous la table, la grotte sent le bois.
-copain|Tu es passée, moi je gardais.
+copain|Tu es passée, moi je fouettais.
 enfant-f|Tes épaules l'ont laissé ouvert.
 papa|Vous l'avez, enfin.
-maman|La cuillère dort sur le bord, au calme.
+maman|La petite tasse dort sur le bord, au calme.
 narrateur|Le bidon de cacao couvre encore leurs genoux.
 enfant-f|On reste un peu, Victorino.
 narrateur|Un rai brun s'endort sous le bois.
-narrateur|La poussière redevient douce, autour.</t>
+narrateur|La miette redevient douce, autour.</t>
         </is>
       </c>
     </row>
@@ -5872,12 +5872,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>On écarte un peu. Moi aussi, j'écarte. Victorino tire la chaise, tout haut. Nina se glisse, pendant l'ouverture. Le bidon soulève la poussière, tout doux. Il est venu vers vous. On l'a repris. Il fume encore. Vos cheveux sentent le bois chaud.</t>
+          <t>On écarte la chaise. Moi aussi, j'écarte. Victorino tire la chaise, tout haut. Nina se glisse, pendant l'ouverture. Le bidon avance, tout doux, vers le jour. La place est venue vers vous. Je rentre, de côté. On y est, tous les deux. Vos cheveux sentent le bois chaud.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>On écarte un peu. Moi aussi, j'écarte. Victorino tire la chaise, tout haut. Nina se glisse, pendant l'ouverture. Le bidon soulève la poussière, tout doux. Il est venu vers vous. On l'a repris. Il fume encore. Vos cheveux sentent le bois chaud.</t>
+          <t>On écarte la chaise. Moi aussi, j'écarte. Victorino tire la chaise, tout haut. Nina se glisse, pendant l'ouverture. Le bidon avance, tout doux, vers le jour. La place est venue vers vous. Je rentre, de côté. On y est, tous les deux. Vos cheveux sentent le bois chaud.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -6012,14 +6012,14 @@
       <c r="AV28" s="2" t="inlineStr"/>
       <c r="AW28" t="inlineStr">
         <is>
-          <t>enfant-f|On écarte un peu.
+          <t>enfant-f|On écarte la chaise.
 copain|Moi aussi, j'écarte.
 narrateur|Victorino tire la chaise, tout haut.
 narrateur|Nina se glisse, pendant l'ouverture.
-narrateur|Le bidon soulève la poussière, tout doux.
-papa|Il est venu vers vous.
-copain|On l'a repris.
-enfant-f|Il fume encore.
+narrateur|Le bidon avance, tout doux, vers le jour.
+papa|La place est venue vers vous.
+copain|Je rentre, de côté.
+enfant-f|On y est, tous les deux.
 maman|Vos cheveux sentent le bois chaud.</t>
         </is>
       </c>
@@ -6047,12 +6047,12 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Le bord de table redescend, tout doux. Il est tombé vers nous. On a écarté, tous les deux. Il n'était plus trop coincé. La poudre froisse encore, dans l'air. Le bidon de cacao retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des chaises. Le radiateur se tait, contre le mur.</t>
+          <t>Le bord de table redescend, tout doux. Je suis rentré de côté. On a écarté, tous les deux. Il n'était plus trop coincé. La poudre danse encore, dans l'air. Le bidon de cacao retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des chaises. Le radiateur se tait, contre le mur.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Le bord de table redescend, tout doux. Il est tombé vers nous. On a écarté, tous les deux. Il n'était plus trop coincé. La poudre froisse encore, dans l'air. Le bidon de cacao retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des chaises. Le radiateur se tait, contre le mur.</t>
+          <t>Le bord de table redescend, tout doux. Je suis rentré de côté. On a écarté, tous les deux. Il n'était plus trop coincé. La poudre danse encore, dans l'air. Le bidon de cacao retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des chaises. Le radiateur se tait, contre le mur.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -6188,10 +6188,10 @@
       <c r="AW29" t="inlineStr">
         <is>
           <t>narrateur|Le bord de table redescend, tout doux.
-copain|Il est tombé vers nous.
+copain|Je suis rentré de côté.
 enfant-f|On a écarté, tous les deux.
 maman|Il n'était plus trop coincé.
-papa|La poudre froisse encore, dans l'air.
+papa|La poudre danse encore, dans l'air.
 narrateur|Le bidon de cacao retombe, tout léger.
 enfant-f|On souffle dessus, tout calme.
 narrateur|Un rayon veille près des chaises.
@@ -6222,12 +6222,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Papa, écarte un peu ? Je fais un chemin, tout doux. Une chaise s'ouvre, comme une aile. Nina rentre, Victorino reste dehors. Le bidon devient un nid, contre le bois. On se parle à travers. Oui. Vous y arrivez, tous les deux. Deux voix tiennent le même secret.</t>
+          <t>Papa, écarte un peu ? Je fais un chemin, tout doux. Une chaise s'ouvre, comme une aile. Nina rentre, Victorino reste dehors. Le bidon devient un nid, contre le bois. On trinque à travers ? Oui, petite tasse, grande tasse. Vous y arrivez, tous les deux. Deux voix tiennent le même secret.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Papa, écarte un peu ? Je fais un chemin, tout doux. Une chaise s'ouvre, comme une aile. Nina rentre, Victorino reste dehors. Le bidon devient un nid, contre le bois. On se parle à travers. Oui. Vous y arrivez, tous les deux. Deux voix tiennent le même secret.</t>
+          <t>Papa, écarte un peu ? Je fais un chemin, tout doux. Une chaise s'ouvre, comme une aile. Nina rentre, Victorino reste dehors. Le bidon devient un nid, contre le bois. On trinque à travers ? Oui, petite tasse, grande tasse. Vous y arrivez, tous les deux. Deux voix tiennent le même secret.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -6367,8 +6367,8 @@
 narrateur|Une chaise s'ouvre, comme une aile.
 narrateur|Nina rentre, Victorino reste dehors.
 narrateur|Le bidon devient un nid, contre le bois.
-copain|On se parle à travers.
-enfant-f|Oui.
+copain|On trinque à travers ?
+enfant-f|Oui, petite tasse, grande tasse.
 maman|Vous y arrivez, tous les deux.
 narrateur|Deux voix tiennent le même secret.</t>
         </is>
@@ -6397,12 +6397,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Deux têtes se parlent encore, à travers le bois. On s'est parlé à travers. La table vous a laissé la place. Le secret tient encore, tout chaud. Le bidon de cacao garde un brin de lait. Regarde-le, Victorino, il fume. Je le vois, d'ici. Le brun reste au chaud, sous le bois. Une chaise redevient calme, tout seule.</t>
+          <t>Deux tasses se parlent encore, à travers le bois. On a trinqué à travers. La table vous a laissé la place. Le secret tient encore, tout chaud. Le bidon de cacao garde un brin de lait. Regarde-le, Victorino, il fume. Je le vois, d'ici. Le brun reste au chaud, sous le bois. Une chaise redevient calme, tout seule.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Deux têtes se parlent encore, à travers le bois. On s'est parlé à travers. La table vous a laissé la place. Le secret tient encore, tout chaud. Le bidon de cacao garde un brin de lait. Regarde-le, Victorino, il fume. Je le vois, d'ici. Le brun reste au chaud, sous le bois. Une chaise redevient calme, tout seule.</t>
+          <t>Deux tasses se parlent encore, à travers le bois. On a trinqué à travers. La table vous a laissé la place. Le secret tient encore, tout chaud. Le bidon de cacao garde un brin de lait. Regarde-le, Victorino, il fume. Je le vois, d'ici. Le brun reste au chaud, sous le bois. Une chaise redevient calme, tout seule.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -6537,8 +6537,8 @@
       <c r="AV31" s="2" t="inlineStr"/>
       <c r="AW31" t="inlineStr">
         <is>
-          <t>narrateur|Deux têtes se parlent encore, à travers le bois.
-copain|On s'est parlé à travers.
+          <t>narrateur|Deux tasses se parlent encore, à travers le bois.
+copain|On a trinqué à travers.
 papa|La table vous a laissé la place.
 maman|Le secret tient encore, tout chaud.
 narrateur|Le bidon de cacao garde un brin de lait.
@@ -6934,12 +6934,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>La poche veille près du fouet. J'entends le clic ! Ne le sors pas encore. Victorino a les cheveux tout courts. Une mèche saute quand il se baisse. Ça sent déjà le cacao, sur le métal. Vos mains, au-dessus du plateau ? Oui, maman.</t>
+          <t>La poche veille près du fouet. J'entends le clic ! Ne le sors pas encore. Victorino se baisse, trop long, trop vite. Une mèche saute au-dessus du pichet. Ça sent déjà le cacao, sur le métal. Vos mains, au-dessus du plateau ? Oui, maman.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>La poche veille près du fouet. J'entends le clic ! Ne le sors pas encore. Victorino a les cheveux tout courts. Une mèche saute quand il se baisse. Ça sent déjà le cacao, sur le métal. Vos mains, au-dessus du plateau ? Oui, maman.</t>
+          <t>La poche veille près du fouet. J'entends le clic ! Ne le sors pas encore. Victorino se baisse, trop long, trop vite. Une mèche saute au-dessus du pichet. Ça sent déjà le cacao, sur le métal. Vos mains, au-dessus du plateau ? Oui, maman.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -7081,8 +7081,8 @@
           <t>narrateur|La poche veille près du fouet.
 copain|J'entends le clic !
 enfant-f|Ne le sors pas encore.
-narrateur|Victorino a les cheveux tout courts.
-narrateur|Une mèche saute quand il se baisse.
+narrateur|Victorino se baisse, trop long, trop vite.
+narrateur|Une mèche saute au-dessus du pichet.
 papa|Ça sent déjà le cacao, sur le métal.
 maman|Vos mains, au-dessus du plateau ?
 copain|Oui, maman.</t>
@@ -7307,12 +7307,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Le fouet tape une planche, toc. Le plan de travail sent le citron, trop haut. Moi je vois le fond du bol ! Victorino se hausse, trop vite. Ses doigts trouvent déjà le rebord froid. Le clic de métal se perd entre les bols. Le fouet n'attendait pas ça. Tes bras n'arrivent pas encore. Lui voit le haut, toi le bois. On mélange comment, alors ? Vous faites comment, tous les deux ?</t>
+          <t>Nina pose le fouet sur le plan, trop haut. Le grand bol attend, trop loin pour Nina. Je ne vois plus le fond. Moi si, il est tout brun. Victorino se hausse, le menton au rebord. Les fils du fouet disparaissent derrière le bol. Le fouet reste au-dessus d'elle, trop loin. Ses bras vont jusqu'au bol. Toi tu vois le bois, lui la poudre. On mélange comment, alors ? Vous faites comment, tous les deux ?</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Le fouet tape une planche, toc. Le plan de travail sent le citron, trop haut. Moi je vois le fond du bol ! Victorino se hausse, trop vite. Ses doigts trouvent déjà le rebord froid. Le clic de métal se perd entre les bols. Le fouet n'attendait pas ça. Tes bras n'arrivent pas encore. Lui voit le haut, toi le bois. On mélange comment, alors ? Vous faites comment, tous les deux ?</t>
+          <t>Nina pose le fouet sur le plan, trop haut. Le grand bol attend, trop loin pour Nina. Je ne vois plus le fond. Moi si, il est tout brun. Victorino se hausse, le menton au rebord. Les fils du fouet disparaissent derrière le bol. Le fouet reste au-dessus d'elle, trop loin. Ses bras vont jusqu'au bol. Toi tu vois le bois, lui la poudre. On mélange comment, alors ? Vous faites comment, tous les deux ?</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -7447,16 +7447,16 @@
       <c r="AV36" s="2" t="inlineStr"/>
       <c r="AW36" t="inlineStr">
         <is>
-          <t>narrateur|Le fouet tape une planche, toc.
-narrateur|Le plan de travail sent le citron, trop haut.
-copain|Moi je vois le fond du bol !
-narrateur|Victorino se hausse, trop vite.
-narrateur|Ses doigts trouvent déjà le rebord froid.
-narrateur|Le clic de métal se perd entre les bols.
-enfant-f|Le fouet n'attendait pas ça.
-maman|Tes bras n'arrivent pas encore.
-papa|Lui voit le haut, toi le bois.
-copain|On mélange comment, alors ?
+          <t>narrateur|Nina pose le fouet sur le plan, trop haut.
+narrateur|Le grand bol attend, trop loin pour Nina.
+enfant-f|Je ne vois plus le fond.
+copain|Moi si, il est tout brun.
+narrateur|Victorino se hausse, le menton au rebord.
+narrateur|Les fils du fouet disparaissent derrière le bol.
+narrateur|Le fouet reste au-dessus d'elle, trop loin.
+maman|Ses bras vont jusqu'au bol.
+papa|Toi tu vois le bois, lui la poudre.
+enfant-f|On mélange comment, alors ?
 papa|Vous faites comment, tous les deux ?</t>
         </is>
       </c>
@@ -7680,12 +7680,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Tu mélanges, Victorino. Victorino lève le bol, assez haut. Doucement. Nina tend le fouet, bras tout courts. Ses doigts trouvent un rebord froid. Je tiens le bas ! Tes bras allaient assez loin. La poudre s'ouvre, à leur hauteur. Regarde, Nina. Il est à nous.</t>
+          <t>Tu mélanges, toi, tu vois le fond. Victorino tourne dans le bol, assez haut. Ça devient brun, tout doux. Nina tend le fouet, bras tout courts. Nina verse le lait, d'en bas, tout lent. Je tiens le pichet ! Tes bras allaient assez loin. La poudre s'ouvre, à leur hauteur. Goûte, Nina. Il est à nous.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Tu mélanges, Victorino. Victorino lève le bol, assez haut. Doucement. Nina tend le fouet, bras tout courts. Ses doigts trouvent un rebord froid. Je tiens le bas ! Tes bras allaient assez loin. La poudre s'ouvre, à leur hauteur. Regarde, Nina. Il est à nous.</t>
+          <t>Tu mélanges, toi, tu vois le fond. Victorino tourne dans le bol, assez haut. Ça devient brun, tout doux. Nina tend le fouet, bras tout courts. Nina verse le lait, d'en bas, tout lent. Je tiens le pichet ! Tes bras allaient assez loin. La poudre s'ouvre, à leur hauteur. Goûte, Nina. Il est à nous.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -7820,15 +7820,15 @@
       <c r="AV38" s="2" t="inlineStr"/>
       <c r="AW38" t="inlineStr">
         <is>
-          <t>enfant-f|Tu mélanges, Victorino.
-narrateur|Victorino lève le bol, assez haut.
-copain|Doucement.
+          <t>enfant-f|Tu mélanges, toi, tu vois le fond.
+narrateur|Victorino tourne dans le bol, assez haut.
+copain|Ça devient brun, tout doux.
 narrateur|Nina tend le fouet, bras tout courts.
-narrateur|Ses doigts trouvent un rebord froid.
-enfant-f|Je tiens le bas !
+narrateur|Nina verse le lait, d'en bas, tout lent.
+enfant-f|Je tiens le pichet !
 papa|Tes bras allaient assez loin.
 narrateur|La poudre s'ouvre, à leur hauteur.
-copain|Regarde, Nina.
+copain|Goûte, Nina.
 enfant-f|Il est à nous.</t>
         </is>
       </c>
@@ -7856,12 +7856,12 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>À l'étagère, le cacao sent le citron. Tu tenais le bas, moi je mélangeais. Tes bras l'ont fait monter. Vous l'avez, enfin. Le bol dort sur le bois, au calme. Le fouet veille encore au bas. On reste un peu, Victorino. Un rai brun s'endort sur les carreaux. La buée redevient douce, dans l'air.</t>
+          <t>À l'étagère, le cacao sent le citron. Tu versais, moi je tournais. Tes bras ont vu le fond. Vous l'avez, enfin. Le bol dort sur le bois, au calme. Le fouet veille encore au bas, un peu brun. On reste un peu, Victorino. Un rai brun s'endort sur les carreaux. La buée redevient douce, dans l'air.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>À l'étagère, le cacao sent le citron. Tu tenais le bas, moi je mélangeais. Tes bras l'ont fait monter. Vous l'avez, enfin. Le bol dort sur le bois, au calme. Le fouet veille encore au bas. On reste un peu, Victorino. Un rai brun s'endort sur les carreaux. La buée redevient douce, dans l'air.</t>
+          <t>À l'étagère, le cacao sent le citron. Tu versais, moi je tournais. Tes bras ont vu le fond. Vous l'avez, enfin. Le bol dort sur le bois, au calme. Le fouet veille encore au bas, un peu brun. On reste un peu, Victorino. Un rai brun s'endort sur les carreaux. La buée redevient douce, dans l'air.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -7997,11 +7997,11 @@
       <c r="AW39" t="inlineStr">
         <is>
           <t>narrateur|À l'étagère, le cacao sent le citron.
-copain|Tu tenais le bas, moi je mélangeais.
-enfant-f|Tes bras l'ont fait monter.
+copain|Tu versais, moi je tournais.
+enfant-f|Tes bras ont vu le fond.
 papa|Vous l'avez, enfin.
 maman|Le bol dort sur le bois, au calme.
-narrateur|Le fouet veille encore au bas.
+narrateur|Le fouet veille encore au bas, un peu brun.
 enfant-f|On reste un peu, Victorino.
 narrateur|Un rai brun s'endort sur les carreaux.
 narrateur|La buée redevient douce, dans l'air.</t>
@@ -8031,12 +8031,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Je monte, tout doux. Tiens le bois, Nina. Nina se hausse, plus petite que le bol. Moi je guide, tout près. Victorino tient le lait, au-dessus. La poudre glisse vers le fond. Il est à toi, un moment. Vous le partagez. Le fouet attend au bord, un peu rêche.</t>
+          <t>Je monte, tout doux. Tiens le bois, Nina. Nina se hausse, le nez au bord du bol. Moi je verse le lait, tout près. Victorino tient le pichet, au-dessus. La poudre glisse vers le fond. Tu vois, maintenant. Vous le partagez. Le fouet attend au bord, un peu rêche.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Je monte, tout doux. Tiens le bois, Nina. Nina se hausse, plus petite que le bol. Moi je guide, tout près. Victorino tient le lait, au-dessus. La poudre glisse vers le fond. Il est à toi, un moment. Vous le partagez. Le fouet attend au bord, un peu rêche.</t>
+          <t>Je monte, tout doux. Tiens le bois, Nina. Nina se hausse, le nez au bord du bol. Moi je verse le lait, tout près. Victorino tient le pichet, au-dessus. La poudre glisse vers le fond. Tu vois, maintenant. Vous le partagez. Le fouet attend au bord, un peu rêche.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -8173,11 +8173,11 @@
         <is>
           <t>enfant-f|Je monte, tout doux.
 papa|Tiens le bois, Nina.
-narrateur|Nina se hausse, plus petite que le bol.
-copain|Moi je guide, tout près.
-narrateur|Victorino tient le lait, au-dessus.
+narrateur|Nina se hausse, le nez au bord du bol.
+copain|Moi je verse le lait, tout près.
+narrateur|Victorino tient le pichet, au-dessus.
 narrateur|La poudre glisse vers le fond.
-copain|Il est à toi, un moment.
+copain|Tu vois, maintenant.
 maman|Vous le partagez.
 narrateur|Le fouet attend au bord, un peu rêche.</t>
         </is>
@@ -8206,12 +8206,12 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Sur le tabouret, deux têtes se calment. Victorino, tu l'as vue glisser. Oui, tout près de tes mains. Toi en bas, lui au-dessus, ça tenait. Vos voix sont devenues toutes petites. Le fouet reste dans la paume de Nina. Je reste encore un peu. Une goutte reste collée au bol. L'évier sent encore le cacao.</t>
+          <t>Sur le tabouret, deux têtes se calment. J'ai vu le fond, moi aussi. Oui, tu étais assez haute. Toi en bas, lui au-dessus, ça tenait. Vos voix sont devenues toutes petites. Le fouet reste dans la paume de Nina. Je reste encore un peu. Une goutte reste collée au bol. L'évier sent encore le cacao.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Sur le tabouret, deux têtes se calment. Victorino, tu l'as vue glisser. Oui, tout près de tes mains. Toi en bas, lui au-dessus, ça tenait. Vos voix sont devenues toutes petites. Le fouet reste dans la paume de Nina. Je reste encore un peu. Une goutte reste collée au bol. L'évier sent encore le cacao.</t>
+          <t>Sur le tabouret, deux têtes se calment. J'ai vu le fond, moi aussi. Oui, tu étais assez haute. Toi en bas, lui au-dessus, ça tenait. Vos voix sont devenues toutes petites. Le fouet reste dans la paume de Nina. Je reste encore un peu. Une goutte reste collée au bol. L'évier sent encore le cacao.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -8347,8 +8347,8 @@
       <c r="AW41" t="inlineStr">
         <is>
           <t>narrateur|Sur le tabouret, deux têtes se calment.
-enfant-f|Victorino, tu l'as vue glisser.
-copain|Oui, tout près de tes mains.
+enfant-f|J'ai vu le fond, moi aussi.
+copain|Oui, tu étais assez haute.
 papa|Toi en bas, lui au-dessus, ça tenait.
 maman|Vos voix sont devenues toutes petites.
 narrateur|Le fouet reste dans la paume de Nina.
@@ -8381,12 +8381,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>On tire un peu. Moi aussi, je tire. Victorino lève un torchon, tout haut. Nina glisse le bol, pendant l'ouverture. Le fouet accroche le torchon, clic. Il est venu vers vous. On l'a repris. Il fume encore. Vos cheveux sentent le linge chaud.</t>
+          <t>On tire le bol, tout doux. Moi aussi, je tire. Victorino enroule un torchon, tout haut. Nina tire l'autre bout, plus bas. Le fouet glisse avec le torchon, clic. Le bol est venu vers vous. On le tient. Il fume encore. Vos cheveux sentent le linge chaud.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>On tire un peu. Moi aussi, je tire. Victorino lève un torchon, tout haut. Nina glisse le bol, pendant l'ouverture. Le fouet accroche le torchon, clic. Il est venu vers vous. On l'a repris. Il fume encore. Vos cheveux sentent le linge chaud.</t>
+          <t>On tire le bol, tout doux. Moi aussi, je tire. Victorino enroule un torchon, tout haut. Nina tire l'autre bout, plus bas. Le fouet glisse avec le torchon, clic. Le bol est venu vers vous. On le tient. Il fume encore. Vos cheveux sentent le linge chaud.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -8521,13 +8521,13 @@
       <c r="AV42" s="2" t="inlineStr"/>
       <c r="AW42" t="inlineStr">
         <is>
-          <t>enfant-f|On tire un peu.
+          <t>enfant-f|On tire le bol, tout doux.
 copain|Moi aussi, je tire.
-narrateur|Victorino lève un torchon, tout haut.
-narrateur|Nina glisse le bol, pendant l'ouverture.
-narrateur|Le fouet accroche le torchon, clic.
-papa|Il est venu vers vous.
-copain|On l'a repris.
+narrateur|Victorino enroule un torchon, tout haut.
+narrateur|Nina tire l'autre bout, plus bas.
+narrateur|Le fouet glisse avec le torchon, clic.
+papa|Le bol est venu vers vous.
+copain|On le tient.
 enfant-f|Il fume encore.
 maman|Vos cheveux sentent le linge chaud.</t>
         </is>
@@ -8556,12 +8556,12 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Le torchon redescend, tout doux. Il est tombé vers nous. On a tiré, tous les deux. Il n'était plus trop coincé. La poudre froisse encore, dans l'air. Le fouet retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des bols. Le radiateur se tait, au fond.</t>
+          <t>Le torchon redescend, tout doux. Le bol est venu vers nous. On a tiré, tous les deux. Il n'était plus trop haut. La poudre danse encore, dans l'air. Le fouet retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des bols. Le radiateur se tait, au fond.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Le torchon redescend, tout doux. Il est tombé vers nous. On a tiré, tous les deux. Il n'était plus trop coincé. La poudre froisse encore, dans l'air. Le fouet retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des bols. Le radiateur se tait, au fond.</t>
+          <t>Le torchon redescend, tout doux. Le bol est venu vers nous. On a tiré, tous les deux. Il n'était plus trop haut. La poudre danse encore, dans l'air. Le fouet retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des bols. Le radiateur se tait, au fond.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -8697,10 +8697,10 @@
       <c r="AW43" t="inlineStr">
         <is>
           <t>narrateur|Le torchon redescend, tout doux.
-copain|Il est tombé vers nous.
+copain|Le bol est venu vers nous.
 enfant-f|On a tiré, tous les deux.
-maman|Il n'était plus trop coincé.
-papa|La poudre froisse encore, dans l'air.
+maman|Il n'était plus trop haut.
+papa|La poudre danse encore, dans l'air.
 narrateur|Le fouet retombe, tout léger.
 enfant-f|On souffle dessus, tout calme.
 narrateur|Un rayon veille près des bols.
@@ -8731,12 +8731,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Le fouet glisse vers la poignée, trop vite. Le lait est à nous, Victorino. Je vois le beurre, tout haut ! La poignée reste trop loin pour Nina. Le clic n'atteint pas encore le loquet. Un peu d'air froid lève, puis retombe. Ses bras vont jusqu'à la poignée. Toi tu vois le bac, lui le beurre. On peut jouer avec lui ? Vous trouvez, tous les deux ?</t>
+          <t>Nina tape le fouet contre la porte, toc. Le lait est dedans, Victorino. Je vois déjà le beurre, tout haut ! La poignée reste trop loin pour Nina. Le fouet n'accroche pas encore le loquet. Un souffle froid lève, puis retombe. Ses bras vont jusqu'à la poignée. Toi tu vois le bac, lui le beurre. On ouvre comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Le fouet glisse vers la poignée, trop vite. Le lait est à nous, Victorino. Je vois le beurre, tout haut ! La poignée reste trop loin pour Nina. Le clic n'atteint pas encore le loquet. Un peu d'air froid lève, puis retombe. Ses bras vont jusqu'à la poignée. Toi tu vois le bac, lui le beurre. On peut jouer avec lui ? Vous trouvez, tous les deux ?</t>
+          <t>Nina tape le fouet contre la porte, toc. Le lait est dedans, Victorino. Je vois déjà le beurre, tout haut ! La poignée reste trop loin pour Nina. Le fouet n'accroche pas encore le loquet. Un souffle froid lève, puis retombe. Ses bras vont jusqu'à la poignée. Toi tu vois le bac, lui le beurre. On ouvre comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -8871,15 +8871,15 @@
       <c r="AV44" s="2" t="inlineStr"/>
       <c r="AW44" t="inlineStr">
         <is>
-          <t>narrateur|Le fouet glisse vers la poignée, trop vite.
-enfant-f|Le lait est à nous, Victorino.
-copain|Je vois le beurre, tout haut !
+          <t>narrateur|Nina tape le fouet contre la porte, toc.
+enfant-f|Le lait est dedans, Victorino.
+copain|Je vois déjà le beurre, tout haut !
 narrateur|La poignée reste trop loin pour Nina.
-narrateur|Le clic n'atteint pas encore le loquet.
-narrateur|Un peu d'air froid lève, puis retombe.
+narrateur|Le fouet n'accroche pas encore le loquet.
+narrateur|Un souffle froid lève, puis retombe.
 maman|Ses bras vont jusqu'à la poignée.
 papa|Toi tu vois le bac, lui le beurre.
-enfant-f|On peut jouer avec lui ?
+enfant-f|On ouvre comment, alors ?
 papa|Vous trouvez, tous les deux ?</t>
         </is>
       </c>
@@ -9103,12 +9103,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Je me hausse encore. Je tiens les tasses, d'en bas. Les doigts de Victorino touchent la poignée. Elle bouge ! Le lait penche, puis avance. Victorino pose le fouet contre la porte. Tes doigts allaient assez loin. Nina tenait bien le bas. Il est à nous.</t>
+          <t>Je me hausse encore. Je tiens les tasses, d'en bas. Les doigts de Victorino touchent la poignée. Elle bouge ! La bouteille de lait penche, puis avance. Victorino pose le fouet contre la porte. Tes doigts allaient assez loin. Nina tenait bien le bas. Le lait est à nous.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Je me hausse encore. Je tiens les tasses, d'en bas. Les doigts de Victorino touchent la poignée. Elle bouge ! Le lait penche, puis avance. Victorino pose le fouet contre la porte. Tes doigts allaient assez loin. Nina tenait bien le bas. Il est à nous.</t>
+          <t>Je me hausse encore. Je tiens les tasses, d'en bas. Les doigts de Victorino touchent la poignée. Elle bouge ! La bouteille de lait penche, puis avance. Victorino pose le fouet contre la porte. Tes doigts allaient assez loin. Nina tenait bien le bas. Le lait est à nous.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -9247,11 +9247,11 @@
 enfant-f|Je tiens les tasses, d'en bas.
 narrateur|Les doigts de Victorino touchent la poignée.
 copain|Elle bouge !
-narrateur|Le lait penche, puis avance.
+narrateur|La bouteille de lait penche, puis avance.
 narrateur|Victorino pose le fouet contre la porte.
 papa|Tes doigts allaient assez loin.
 maman|Nina tenait bien le bas.
-copain|Il est à nous.</t>
+copain|Le lait est à nous.</t>
         </is>
       </c>
     </row>
@@ -9278,12 +9278,12 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Au frigo, le cacao sent le lait. Tu l'as fait pencher pour moi. Tu tenais le bas. Le verre sent encore le matin. Le cacao est à vous, maintenant. Le fouet garde un brin de froid. Nina le verse contre la tasse petite. Un rai traverse la vapeur, tout chaud. Le loquet redevient calme, tout seul.</t>
+          <t>Au frigo, le cacao sent le lait. Tu as ouvert, tout haut. Tu tenais les tasses. Le verre sent encore le matin. Le cacao est à vous, maintenant. Le fouet garde un brin de froid. Nina verse dans la tasse petite. Un rai traverse la vapeur, tout chaud. Le loquet redevient calme, tout seul.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Au frigo, le cacao sent le lait. Tu l'as fait pencher pour moi. Tu tenais le bas. Le verre sent encore le matin. Le cacao est à vous, maintenant. Le fouet garde un brin de froid. Nina le verse contre la tasse petite. Un rai traverse la vapeur, tout chaud. Le loquet redevient calme, tout seul.</t>
+          <t>Au frigo, le cacao sent le lait. Tu as ouvert, tout haut. Tu tenais les tasses. Le verre sent encore le matin. Le cacao est à vous, maintenant. Le fouet garde un brin de froid. Nina verse dans la tasse petite. Un rai traverse la vapeur, tout chaud. Le loquet redevient calme, tout seul.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -9419,12 +9419,12 @@
       <c r="AW47" t="inlineStr">
         <is>
           <t>narrateur|Au frigo, le cacao sent le lait.
-enfant-f|Tu l'as fait pencher pour moi.
-copain|Tu tenais le bas.
+enfant-f|Tu as ouvert, tout haut.
+copain|Tu tenais les tasses.
 maman|Le verre sent encore le matin.
 papa|Le cacao est à vous, maintenant.
 narrateur|Le fouet garde un brin de froid.
-narrateur|Nina le verse contre la tasse petite.
+narrateur|Nina verse dans la tasse petite.
 narrateur|Un rai traverse la vapeur, tout chaud.
 narrateur|Le loquet redevient calme, tout seul.</t>
         </is>
@@ -9453,12 +9453,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>J'ouvre le bac du bas ? Oui, tout doux. Nina pose le fouet près du bac. Papa tient la porte, tout ferme. Nina tire le bac, Victorino veille. Le lait est là ! Je le sens. Vous avez regardé ensemble. Le bac est resté doux.</t>
+          <t>J'ouvre le bac du bas ? Oui, tout doux. Nina pose le fouet près du bac. Papa tient la porte, tout ferme. Nina tire le bac, Victorino veille. Le lait est là ! Il est tout froid. Vous avez regardé ensemble. Le bac est resté doux.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>J'ouvre le bac du bas ? Oui, tout doux. Nina pose le fouet près du bac. Papa tient la porte, tout ferme. Nina tire le bac, Victorino veille. Le lait est là ! Je le sens. Vous avez regardé ensemble. Le bac est resté doux.</t>
+          <t>J'ouvre le bac du bas ? Oui, tout doux. Nina pose le fouet près du bac. Papa tient la porte, tout ferme. Nina tire le bac, Victorino veille. Le lait est là ! Il est tout froid. Vous avez regardé ensemble. Le bac est resté doux.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -9599,7 +9599,7 @@
 narrateur|Papa tient la porte, tout ferme.
 narrateur|Nina tire le bac, Victorino veille.
 enfant-f|Le lait est là !
-copain|Je le sens.
+copain|Il est tout froid.
 maman|Vous avez regardé ensemble.
 papa|Le bac est resté doux.</t>
         </is>
@@ -9628,12 +9628,12 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Près du bac, deux paires de pieds se touchent. Tu l'as posé, d'en bas. Tes bras l'ont fait descendre. Chacun a fait sa part, à sa hauteur. Le bois du bac sèche déjà. Le fouet pose une ombre au bac. Il fume trop, Nina. C'est pour ça. La porte garde le froid, tout proche.</t>
+          <t>Près du bac, deux paires de pieds se touchent. Tu l'as trouvé, d'en bas. Tes yeux gardaient la porte. Chacun a fait sa part, à sa hauteur. Le bois du bac sèche déjà. Le fouet pose une ombre au bac. Il fume trop, Nina. C'est pour ça. La porte garde le froid, tout proche.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Près du bac, deux paires de pieds se touchent. Tu l'as posé, d'en bas. Tes bras l'ont fait descendre. Chacun a fait sa part, à sa hauteur. Le bois du bac sèche déjà. Le fouet pose une ombre au bac. Il fume trop, Nina. C'est pour ça. La porte garde le froid, tout proche.</t>
+          <t>Près du bac, deux paires de pieds se touchent. Tu l'as trouvé, d'en bas. Tes yeux gardaient la porte. Chacun a fait sa part, à sa hauteur. Le bois du bac sèche déjà. Le fouet pose une ombre au bac. Il fume trop, Nina. C'est pour ça. La porte garde le froid, tout proche.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -9769,8 +9769,8 @@
       <c r="AW49" t="inlineStr">
         <is>
           <t>narrateur|Près du bac, deux paires de pieds se touchent.
-copain|Tu l'as posé, d'en bas.
-enfant-f|Tes bras l'ont fait descendre.
+copain|Tu l'as trouvé, d'en bas.
+enfant-f|Tes yeux gardaient la porte.
 papa|Chacun a fait sa part, à sa hauteur.
 maman|Le bois du bac sèche déjà.
 narrateur|Le fouet pose une ombre au bac.
@@ -9803,12 +9803,12 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Reste en haut, Victorino. Je tends, d'ici. Victorino tend le fouet, bras tout longs. Victorino fait basculer le loquet, tout doux. Le tabouret prend Nina, puis lui. Je le tiens ! Chacun a fait sa part. Il sent le froid. Vos bras n'avaient pas la même longueur.</t>
+          <t>Reste en haut, Victorino. Je tends, d'ici. Victorino tend le fouet, bras tout longs. Victorino fait basculer le loquet, tout doux. Le tabouret prend Nina, puis lui. Je tiens la bouteille ! Chacun a fait sa part. Elle sent le froid. Vos bras n'avaient pas la même longueur.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Reste en haut, Victorino. Je tends, d'ici. Victorino tend le fouet, bras tout longs. Victorino fait basculer le loquet, tout doux. Le tabouret prend Nina, puis lui. Je le tiens ! Chacun a fait sa part. Il sent le froid. Vos bras n'avaient pas la même longueur.</t>
+          <t>Reste en haut, Victorino. Je tends, d'ici. Victorino tend le fouet, bras tout longs. Victorino fait basculer le loquet, tout doux. Le tabouret prend Nina, puis lui. Je tiens la bouteille ! Chacun a fait sa part. Elle sent le froid. Vos bras n'avaient pas la même longueur.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -9948,9 +9948,9 @@
 narrateur|Victorino tend le fouet, bras tout longs.
 narrateur|Victorino fait basculer le loquet, tout doux.
 narrateur|Le tabouret prend Nina, puis lui.
-enfant-f|Je le tiens !
+enfant-f|Je tiens la bouteille !
 papa|Chacun a fait sa part.
-copain|Il sent le froid.
+copain|Elle sent le froid.
 maman|Vos bras n'avaient pas la même longueur.</t>
         </is>
       </c>
@@ -9978,12 +9978,12 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Un peu de buée reste au frigo. On a tiré ensemble. Sans trop monter. Le tabouret est resté à sa place. Vos mains sentent encore le lait. Nina pose le fouet au rebord. Tu l'as eu, enfin. Il est à nous. La vapeur tremble un peu, puis s'endort.</t>
+          <t>Un peu de buée reste au frigo. On a ouvert ensemble. Sans trop monter. Le tabouret est resté à sa place. Vos mains sentent encore le lait. Nina pose le fouet au rebord. Tu l'as eu, enfin. Il est à nous. La vapeur tremble un peu, puis s'endort.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Un peu de buée reste au frigo. On a tiré ensemble. Sans trop monter. Le tabouret est resté à sa place. Vos mains sentent encore le lait. Nina pose le fouet au rebord. Tu l'as eu, enfin. Il est à nous. La vapeur tremble un peu, puis s'endort.</t>
+          <t>Un peu de buée reste au frigo. On a ouvert ensemble. Sans trop monter. Le tabouret est resté à sa place. Vos mains sentent encore le lait. Nina pose le fouet au rebord. Tu l'as eu, enfin. Il est à nous. La vapeur tremble un peu, puis s'endort.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -10119,7 +10119,7 @@
       <c r="AW51" t="inlineStr">
         <is>
           <t>narrateur|Un peu de buée reste au frigo.
-enfant-f|On a tiré ensemble.
+enfant-f|On a ouvert ensemble.
 copain|Sans trop monter.
 papa|Le tabouret est resté à sa place.
 maman|Vos mains sentent encore le lait.
@@ -10153,12 +10153,12 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Le fouet roule sous une chaise, toc. Ici, ça sent le bois, Victorino. Je me glisse, trop large ! Ses épaules butent contre le bois de la table. Le clic se perd entre les pieds de chaise. Le fouet attend au bord, un peu seul. Il a les épaules trop larges, c'est tout. Toi tu passes, lui pas encore. On joue comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>Nina glisse le fouet sous la table, tout bas. On goûte ici, comme une grotte. J'entre, trop large ! Ses épaules butent contre le bois de la table. Le fouet roule, puis s'arrête contre un pied. Le fouet attend au bord, un peu seul. Il a les épaules trop larges, c'est tout. Toi tu passes, lui pas encore. On goûte comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Le fouet roule sous une chaise, toc. Ici, ça sent le bois, Victorino. Je me glisse, trop large ! Ses épaules butent contre le bois de la table. Le clic se perd entre les pieds de chaise. Le fouet attend au bord, un peu seul. Il a les épaules trop larges, c'est tout. Toi tu passes, lui pas encore. On joue comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>Nina glisse le fouet sous la table, tout bas. On goûte ici, comme une grotte. J'entre, trop large ! Ses épaules butent contre le bois de la table. Le fouet roule, puis s'arrête contre un pied. Le fouet attend au bord, un peu seul. Il a les épaules trop larges, c'est tout. Toi tu passes, lui pas encore. On goûte comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -10293,15 +10293,15 @@
       <c r="AV52" s="2" t="inlineStr"/>
       <c r="AW52" t="inlineStr">
         <is>
-          <t>narrateur|Le fouet roule sous une chaise, toc.
-enfant-f|Ici, ça sent le bois, Victorino.
-copain|Je me glisse, trop large !
+          <t>narrateur|Nina glisse le fouet sous la table, tout bas.
+enfant-f|On goûte ici, comme une grotte.
+copain|J'entre, trop large !
 narrateur|Ses épaules butent contre le bois de la table.
-narrateur|Le clic se perd entre les pieds de chaise.
+narrateur|Le fouet roule, puis s'arrête contre un pied.
 narrateur|Le fouet attend au bord, un peu seul.
 maman|Il a les épaules trop larges, c'est tout.
 papa|Toi tu passes, lui pas encore.
-copain|On joue comment, alors ?
+copain|On goûte comment, alors ?
 papa|Vous trouvez, tous les deux ?</t>
         </is>
       </c>
@@ -10525,12 +10525,12 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Je passe, Victorino. Nina rampe, tout petite, sous la table. Doucement. Nina glisse le fouet sous le bois. Ses doigts trouvent une cuillère perdue. Je la tiens ! Tes épaules étaient assez petites. Une grotte de lumière s'ouvre, à eux. Regarde, Nina. Elle est à nous.</t>
+          <t>Je passe, toi tu restes. Nina rampe, tout petite, sous la table. Je fouette ici, dehors. Nina glisse le fouet sous le bois. Ses doigts trouvent la petite tasse. Je la tiens ! Tes épaules étaient assez petites. Une grotte de vapeur s'ouvre, à eux. Je te verse, d'ici. Elle est à nous.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Je passe, Victorino. Nina rampe, tout petite, sous la table. Doucement. Nina glisse le fouet sous le bois. Ses doigts trouvent une cuillère perdue. Je la tiens ! Tes épaules étaient assez petites. Une grotte de lumière s'ouvre, à eux. Regarde, Nina. Elle est à nous.</t>
+          <t>Je passe, toi tu restes. Nina rampe, tout petite, sous la table. Je fouette ici, dehors. Nina glisse le fouet sous le bois. Ses doigts trouvent la petite tasse. Je la tiens ! Tes épaules étaient assez petites. Une grotte de vapeur s'ouvre, à eux. Je te verse, d'ici. Elle est à nous.</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -10665,15 +10665,15 @@
       <c r="AV54" s="2" t="inlineStr"/>
       <c r="AW54" t="inlineStr">
         <is>
-          <t>enfant-f|Je passe, Victorino.
+          <t>enfant-f|Je passe, toi tu restes.
 narrateur|Nina rampe, tout petite, sous la table.
-copain|Doucement.
+copain|Je fouette ici, dehors.
 narrateur|Nina glisse le fouet sous le bois.
-narrateur|Ses doigts trouvent une cuillère perdue.
+narrateur|Ses doigts trouvent la petite tasse.
 enfant-f|Je la tiens !
 papa|Tes épaules étaient assez petites.
-narrateur|Une grotte de lumière s'ouvre, à eux.
-copain|Regarde, Nina.
+narrateur|Une grotte de vapeur s'ouvre, à eux.
+copain|Je te verse, d'ici.
 enfant-f|Elle est à nous.</t>
         </is>
       </c>
@@ -10701,12 +10701,12 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Sous la table, la grotte sent le bois. Tu es passée, moi je gardais. Tes épaules l'ont laissé ouvert. Vous l'avez, enfin. La cuillère dort sur le bord, au calme. Le fouet fait un clic, tout bas. On reste un peu, Victorino. Un rai brun s'endort sous le bois. La poussière redevient douce, autour.</t>
+          <t>Sous la table, la grotte sent le bois. Tu es passée, moi je fouettais. Tes épaules l'ont laissé ouvert. Vous l'avez, enfin. La petite tasse dort sur le bord, au calme. Le fouet fait un clic, tout bas. On reste un peu, Victorino. Un rai brun s'endort sous le bois. La miette redevient douce, autour.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Sous la table, la grotte sent le bois. Tu es passée, moi je gardais. Tes épaules l'ont laissé ouvert. Vous l'avez, enfin. La cuillère dort sur le bord, au calme. Le fouet fait un clic, tout bas. On reste un peu, Victorino. Un rai brun s'endort sous le bois. La poussière redevient douce, autour.</t>
+          <t>Sous la table, la grotte sent le bois. Tu es passée, moi je fouettais. Tes épaules l'ont laissé ouvert. Vous l'avez, enfin. La petite tasse dort sur le bord, au calme. Le fouet fait un clic, tout bas. On reste un peu, Victorino. Un rai brun s'endort sous le bois. La miette redevient douce, autour.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -10842,14 +10842,14 @@
       <c r="AW55" t="inlineStr">
         <is>
           <t>narrateur|Sous la table, la grotte sent le bois.
-copain|Tu es passée, moi je gardais.
+copain|Tu es passée, moi je fouettais.
 enfant-f|Tes épaules l'ont laissé ouvert.
 papa|Vous l'avez, enfin.
-maman|La cuillère dort sur le bord, au calme.
+maman|La petite tasse dort sur le bord, au calme.
 narrateur|Le fouet fait un clic, tout bas.
 enfant-f|On reste un peu, Victorino.
 narrateur|Un rai brun s'endort sous le bois.
-narrateur|La poussière redevient douce, autour.</t>
+narrateur|La miette redevient douce, autour.</t>
         </is>
       </c>
     </row>
@@ -10876,12 +10876,12 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>On écarte un peu. Moi aussi, j'écarte. Victorino tire la chaise, tout haut. Nina se glisse, pendant l'ouverture. Le fouet soulève un clic, tout bas. Il est venu vers vous. On l'a repris. Il fume encore. Vos cheveux sentent le bois chaud.</t>
+          <t>On écarte la chaise. Moi aussi, j'écarte. Victorino tire la chaise, tout haut. Nina se glisse, pendant l'ouverture. Le fouet avance, un clic, vers le jour. La place est venue vers vous. Je rentre, de côté. On y est, tous les deux. Vos cheveux sentent le bois chaud.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>On écarte un peu. Moi aussi, j'écarte. Victorino tire la chaise, tout haut. Nina se glisse, pendant l'ouverture. Le fouet soulève un clic, tout bas. Il est venu vers vous. On l'a repris. Il fume encore. Vos cheveux sentent le bois chaud.</t>
+          <t>On écarte la chaise. Moi aussi, j'écarte. Victorino tire la chaise, tout haut. Nina se glisse, pendant l'ouverture. Le fouet avance, un clic, vers le jour. La place est venue vers vous. Je rentre, de côté. On y est, tous les deux. Vos cheveux sentent le bois chaud.</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -11016,14 +11016,14 @@
       <c r="AV56" s="2" t="inlineStr"/>
       <c r="AW56" t="inlineStr">
         <is>
-          <t>enfant-f|On écarte un peu.
+          <t>enfant-f|On écarte la chaise.
 copain|Moi aussi, j'écarte.
 narrateur|Victorino tire la chaise, tout haut.
 narrateur|Nina se glisse, pendant l'ouverture.
-narrateur|Le fouet soulève un clic, tout bas.
-papa|Il est venu vers vous.
-copain|On l'a repris.
-enfant-f|Il fume encore.
+narrateur|Le fouet avance, un clic, vers le jour.
+papa|La place est venue vers vous.
+copain|Je rentre, de côté.
+enfant-f|On y est, tous les deux.
 maman|Vos cheveux sentent le bois chaud.</t>
         </is>
       </c>
@@ -11051,12 +11051,12 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Le bord de table redescend, tout doux. Il est tombé vers nous. On a écarté, tous les deux. Il n'était plus trop coincé. La poudre froisse encore, dans l'air. Le fouet retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des chaises. Le radiateur se tait, contre le mur.</t>
+          <t>Le bord de table redescend, tout doux. Je suis rentré de côté. On a écarté, tous les deux. Il n'était plus trop coincé. La poudre danse encore, dans l'air. Le fouet retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des chaises. Le radiateur se tait, contre le mur.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Le bord de table redescend, tout doux. Il est tombé vers nous. On a écarté, tous les deux. Il n'était plus trop coincé. La poudre froisse encore, dans l'air. Le fouet retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des chaises. Le radiateur se tait, contre le mur.</t>
+          <t>Le bord de table redescend, tout doux. Je suis rentré de côté. On a écarté, tous les deux. Il n'était plus trop coincé. La poudre danse encore, dans l'air. Le fouet retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des chaises. Le radiateur se tait, contre le mur.</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -11192,10 +11192,10 @@
       <c r="AW57" t="inlineStr">
         <is>
           <t>narrateur|Le bord de table redescend, tout doux.
-copain|Il est tombé vers nous.
+copain|Je suis rentré de côté.
 enfant-f|On a écarté, tous les deux.
 maman|Il n'était plus trop coincé.
-papa|La poudre froisse encore, dans l'air.
+papa|La poudre danse encore, dans l'air.
 narrateur|Le fouet retombe, tout léger.
 enfant-f|On souffle dessus, tout calme.
 narrateur|Un rayon veille près des chaises.
@@ -11226,12 +11226,12 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Papa, écarte un peu ? Je fais un chemin, tout doux. Une chaise s'ouvre, comme une aile. Nina rentre, Victorino reste dehors. Le fouet devient un nid, contre le bois. On se parle à travers. Oui. Vous y arrivez, tous les deux. Deux voix tiennent le même secret.</t>
+          <t>Papa, écarte un peu ? Je fais un chemin, tout doux. Une chaise s'ouvre, comme une aile. Nina rentre, Victorino reste dehors. Le fouet devient un nid, contre le bois. On trinque à travers ? Oui, petite tasse, grande tasse. Vous y arrivez, tous les deux. Deux voix tiennent le même secret.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Papa, écarte un peu ? Je fais un chemin, tout doux. Une chaise s'ouvre, comme une aile. Nina rentre, Victorino reste dehors. Le fouet devient un nid, contre le bois. On se parle à travers. Oui. Vous y arrivez, tous les deux. Deux voix tiennent le même secret.</t>
+          <t>Papa, écarte un peu ? Je fais un chemin, tout doux. Une chaise s'ouvre, comme une aile. Nina rentre, Victorino reste dehors. Le fouet devient un nid, contre le bois. On trinque à travers ? Oui, petite tasse, grande tasse. Vous y arrivez, tous les deux. Deux voix tiennent le même secret.</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -11371,8 +11371,8 @@
 narrateur|Une chaise s'ouvre, comme une aile.
 narrateur|Nina rentre, Victorino reste dehors.
 narrateur|Le fouet devient un nid, contre le bois.
-copain|On se parle à travers.
-enfant-f|Oui.
+copain|On trinque à travers ?
+enfant-f|Oui, petite tasse, grande tasse.
 maman|Vous y arrivez, tous les deux.
 narrateur|Deux voix tiennent le même secret.</t>
         </is>
@@ -11401,12 +11401,12 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Deux têtes se parlent encore, à travers le bois. On s'est parlé à travers. La table vous a laissé la place. Le secret tient encore, tout chaud. Le fouet garde un brin de lait. Regarde-le, Victorino, il fume. Je le vois, d'ici. Le brun reste au chaud, sous le bois. Une chaise redevient calme, tout seule.</t>
+          <t>Deux tasses se parlent encore, à travers le bois. On a trinqué à travers. La table vous a laissé la place. Le secret tient encore, tout chaud. Le fouet garde un brin de lait. Regarde-le, Victorino, il fume. Je le vois, d'ici. Le brun reste au chaud, sous le bois. Une chaise redevient calme, tout seule.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Deux têtes se parlent encore, à travers le bois. On s'est parlé à travers. La table vous a laissé la place. Le secret tient encore, tout chaud. Le fouet garde un brin de lait. Regarde-le, Victorino, il fume. Je le vois, d'ici. Le brun reste au chaud, sous le bois. Une chaise redevient calme, tout seule.</t>
+          <t>Deux tasses se parlent encore, à travers le bois. On a trinqué à travers. La table vous a laissé la place. Le secret tient encore, tout chaud. Le fouet garde un brin de lait. Regarde-le, Victorino, il fume. Je le vois, d'ici. Le brun reste au chaud, sous le bois. Une chaise redevient calme, tout seule.</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -11541,8 +11541,8 @@
       <c r="AV59" s="2" t="inlineStr"/>
       <c r="AW59" t="inlineStr">
         <is>
-          <t>narrateur|Deux têtes se parlent encore, à travers le bois.
-copain|On s'est parlé à travers.
+          <t>narrateur|Deux tasses se parlent encore, à travers le bois.
+copain|On a trinqué à travers.
 papa|La table vous a laissé la place.
 maman|Le secret tient encore, tout chaud.
 narrateur|Le fouet garde un brin de lait.
@@ -11938,12 +11938,12 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Le plateau cache encore les deux tasses. Ça sent le lait. Le coin de départ est là. Le pull de Victorino s'arrête trop haut. Les manches laissent ses poignets libres. La cuisine est tiède, autour. On y va, tous les quatre ? Oui.</t>
+          <t>Le plateau cache encore les deux tasses. La grande est à moi ? Oui, la petite est à moi. Le pull de Victorino laisse ses poignets nus. Nina, plus courte, tient le plateau des deux mains. La cuisine est tiède, autour. On y va, tous les quatre ? Oui.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Le plateau cache encore les deux tasses. Ça sent le lait. Le coin de départ est là. Le pull de Victorino s'arrête trop haut. Les manches laissent ses poignets libres. La cuisine est tiède, autour. On y va, tous les quatre ? Oui.</t>
+          <t>Le plateau cache encore les deux tasses. La grande est à moi ? Oui, la petite est à moi. Le pull de Victorino laisse ses poignets nus. Nina, plus courte, tient le plateau des deux mains. La cuisine est tiède, autour. On y va, tous les quatre ? Oui.</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -12083,10 +12083,10 @@
       <c r="AW62" t="inlineStr">
         <is>
           <t>narrateur|Le plateau cache encore les deux tasses.
-copain|Ça sent le lait.
-enfant-f|Le coin de départ est là.
-narrateur|Le pull de Victorino s'arrête trop haut.
-narrateur|Les manches laissent ses poignets libres.
+copain|La grande est à moi ?
+enfant-f|Oui, la petite est à moi.
+narrateur|Le pull de Victorino laisse ses poignets nus.
+narrateur|Nina, plus courte, tient le plateau des deux mains.
 maman|La cuisine est tiède, autour.
 papa|On y va, tous les quatre ?
 enfant-f|Oui.</t>
@@ -12311,12 +12311,12 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Le plateau bute contre l'étagère. Le plan de travail sent le citron, trop haut. Moi je vois le fond du bol ! Victorino se hausse, trop vite. Ses doigts trouvent déjà le rebord froid. Une tasse penche, trop près du vide. Les tasses n'attendait pas ça. Tes bras n'arrivent pas encore. Lui voit le haut, toi le bois. On mélange comment, alors ? Vous faites comment, tous les deux ?</t>
+          <t>Nina pose le plateau sur le plan, trop haut. Le grand bol attend, trop loin pour Nina. Je ne vois plus le fond. Moi si, il est tout brun. Victorino se hausse, le menton au rebord. Les tasses n'arrivent plus, trop basses. Les tasses reste au-dessus d'elle, trop loin. Ses bras vont jusqu'au bol. Toi tu vois le bois, lui la poudre. On mélange comment, alors ? Vous faites comment, tous les deux ?</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Le plateau bute contre l'étagère. Le plan de travail sent le citron, trop haut. Moi je vois le fond du bol ! Victorino se hausse, trop vite. Ses doigts trouvent déjà le rebord froid. Une tasse penche, trop près du vide. Les tasses n'attendait pas ça. Tes bras n'arrivent pas encore. Lui voit le haut, toi le bois. On mélange comment, alors ? Vous faites comment, tous les deux ?</t>
+          <t>Nina pose le plateau sur le plan, trop haut. Le grand bol attend, trop loin pour Nina. Je ne vois plus le fond. Moi si, il est tout brun. Victorino se hausse, le menton au rebord. Les tasses n'arrivent plus, trop basses. Les tasses reste au-dessus d'elle, trop loin. Ses bras vont jusqu'au bol. Toi tu vois le bois, lui la poudre. On mélange comment, alors ? Vous faites comment, tous les deux ?</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -12451,16 +12451,16 @@
       <c r="AV64" s="2" t="inlineStr"/>
       <c r="AW64" t="inlineStr">
         <is>
-          <t>narrateur|Le plateau bute contre l'étagère.
-narrateur|Le plan de travail sent le citron, trop haut.
-copain|Moi je vois le fond du bol !
-narrateur|Victorino se hausse, trop vite.
-narrateur|Ses doigts trouvent déjà le rebord froid.
-narrateur|Une tasse penche, trop près du vide.
-enfant-f|Les tasses n'attendait pas ça.
-maman|Tes bras n'arrivent pas encore.
-papa|Lui voit le haut, toi le bois.
-copain|On mélange comment, alors ?
+          <t>narrateur|Nina pose le plateau sur le plan, trop haut.
+narrateur|Le grand bol attend, trop loin pour Nina.
+enfant-f|Je ne vois plus le fond.
+copain|Moi si, il est tout brun.
+narrateur|Victorino se hausse, le menton au rebord.
+narrateur|Les tasses n'arrivent plus, trop basses.
+narrateur|Les tasses reste au-dessus d'elle, trop loin.
+maman|Ses bras vont jusqu'au bol.
+papa|Toi tu vois le bois, lui la poudre.
+enfant-f|On mélange comment, alors ?
 papa|Vous faites comment, tous les deux ?</t>
         </is>
       </c>
@@ -12684,12 +12684,12 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Tu mélanges, Victorino. Victorino lève le bol, assez haut. Doucement. Nina pousse le plateau, tout près. Ses doigts trouvent un rebord froid. Je tiens le bas ! Tes bras allaient assez loin. La poudre s'ouvre, à leur hauteur. Regarde, Nina. Il est à nous.</t>
+          <t>Tu mélanges, toi, tu vois le fond. Victorino tourne dans le bol, assez haut. Ça devient brun, tout doux. Nina pousse le plateau, tout près. Nina verse le lait, d'en bas, tout lent. Je tiens le pichet ! Tes bras allaient assez loin. La poudre s'ouvre, à leur hauteur. Goûte, Nina. Il est à nous.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Tu mélanges, Victorino. Victorino lève le bol, assez haut. Doucement. Nina pousse le plateau, tout près. Ses doigts trouvent un rebord froid. Je tiens le bas ! Tes bras allaient assez loin. La poudre s'ouvre, à leur hauteur. Regarde, Nina. Il est à nous.</t>
+          <t>Tu mélanges, toi, tu vois le fond. Victorino tourne dans le bol, assez haut. Ça devient brun, tout doux. Nina pousse le plateau, tout près. Nina verse le lait, d'en bas, tout lent. Je tiens le pichet ! Tes bras allaient assez loin. La poudre s'ouvre, à leur hauteur. Goûte, Nina. Il est à nous.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -12824,15 +12824,15 @@
       <c r="AV66" s="2" t="inlineStr"/>
       <c r="AW66" t="inlineStr">
         <is>
-          <t>enfant-f|Tu mélanges, Victorino.
-narrateur|Victorino lève le bol, assez haut.
-copain|Doucement.
+          <t>enfant-f|Tu mélanges, toi, tu vois le fond.
+narrateur|Victorino tourne dans le bol, assez haut.
+copain|Ça devient brun, tout doux.
 narrateur|Nina pousse le plateau, tout près.
-narrateur|Ses doigts trouvent un rebord froid.
-enfant-f|Je tiens le bas !
+narrateur|Nina verse le lait, d'en bas, tout lent.
+enfant-f|Je tiens le pichet !
 papa|Tes bras allaient assez loin.
 narrateur|La poudre s'ouvre, à leur hauteur.
-copain|Regarde, Nina.
+copain|Goûte, Nina.
 enfant-f|Il est à nous.</t>
         </is>
       </c>
@@ -12860,12 +12860,12 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>À l'étagère, le cacao sent le citron. Tu tenais le bas, moi je mélangeais. Tes bras l'ont fait monter. Vous l'avez, enfin. Le bol dort sur le bois, au calme. Le plateau veille encore au bas. On reste un peu, Victorino. Un rai brun s'endort sur les carreaux. La buée redevient douce, dans l'air.</t>
+          <t>À l'étagère, le cacao sent le citron. Tu versais, moi je tournais. Tes bras ont vu le fond. Vous l'avez, enfin. Le bol dort sur le bois, au calme. Le plateau veille encore au bas, deux tasses. On reste un peu, Victorino. Un rai brun s'endort sur les carreaux. La buée redevient douce, dans l'air.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>À l'étagère, le cacao sent le citron. Tu tenais le bas, moi je mélangeais. Tes bras l'ont fait monter. Vous l'avez, enfin. Le bol dort sur le bois, au calme. Le plateau veille encore au bas. On reste un peu, Victorino. Un rai brun s'endort sur les carreaux. La buée redevient douce, dans l'air.</t>
+          <t>À l'étagère, le cacao sent le citron. Tu versais, moi je tournais. Tes bras ont vu le fond. Vous l'avez, enfin. Le bol dort sur le bois, au calme. Le plateau veille encore au bas, deux tasses. On reste un peu, Victorino. Un rai brun s'endort sur les carreaux. La buée redevient douce, dans l'air.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -13001,11 +13001,11 @@
       <c r="AW67" t="inlineStr">
         <is>
           <t>narrateur|À l'étagère, le cacao sent le citron.
-copain|Tu tenais le bas, moi je mélangeais.
-enfant-f|Tes bras l'ont fait monter.
+copain|Tu versais, moi je tournais.
+enfant-f|Tes bras ont vu le fond.
 papa|Vous l'avez, enfin.
 maman|Le bol dort sur le bois, au calme.
-narrateur|Le plateau veille encore au bas.
+narrateur|Le plateau veille encore au bas, deux tasses.
 enfant-f|On reste un peu, Victorino.
 narrateur|Un rai brun s'endort sur les carreaux.
 narrateur|La buée redevient douce, dans l'air.</t>
@@ -13035,12 +13035,12 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Je monte, tout doux. Tiens le bois, Nina. Nina se hausse, plus petite que le bol. Moi je guide, tout près. Victorino tient le lait, au-dessus. La poudre glisse vers le fond. Il est à toi, un moment. Vous le partagez. Le plateau attend au bord, un peu chaud.</t>
+          <t>Je monte, tout doux. Tiens le bois, Nina. Nina se hausse, le nez au bord du bol. Moi je verse le lait, tout près. Victorino tient le pichet, au-dessus. La poudre glisse vers le fond. Tu vois, maintenant. Vous le partagez. Le plateau attend au bord, un peu chaud.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Je monte, tout doux. Tiens le bois, Nina. Nina se hausse, plus petite que le bol. Moi je guide, tout près. Victorino tient le lait, au-dessus. La poudre glisse vers le fond. Il est à toi, un moment. Vous le partagez. Le plateau attend au bord, un peu chaud.</t>
+          <t>Je monte, tout doux. Tiens le bois, Nina. Nina se hausse, le nez au bord du bol. Moi je verse le lait, tout près. Victorino tient le pichet, au-dessus. La poudre glisse vers le fond. Tu vois, maintenant. Vous le partagez. Le plateau attend au bord, un peu chaud.</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13177,11 +13177,11 @@
         <is>
           <t>enfant-f|Je monte, tout doux.
 papa|Tiens le bois, Nina.
-narrateur|Nina se hausse, plus petite que le bol.
-copain|Moi je guide, tout près.
-narrateur|Victorino tient le lait, au-dessus.
+narrateur|Nina se hausse, le nez au bord du bol.
+copain|Moi je verse le lait, tout près.
+narrateur|Victorino tient le pichet, au-dessus.
 narrateur|La poudre glisse vers le fond.
-copain|Il est à toi, un moment.
+copain|Tu vois, maintenant.
 maman|Vous le partagez.
 narrateur|Le plateau attend au bord, un peu chaud.</t>
         </is>
@@ -13210,12 +13210,12 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Sur le tabouret, deux têtes se calment. Victorino, tu l'as vue glisser. Oui, tout près de tes mains. Toi en bas, lui au-dessus, ça tenait. Vos voix sont devenues toutes petites. Les tasses reste dans la paume de Nina. Je reste encore un peu. Une goutte reste collée au bol. L'évier sent encore le cacao.</t>
+          <t>Sur le tabouret, deux têtes se calment. J'ai vu le fond, moi aussi. Oui, tu étais assez haute. Toi en bas, lui au-dessus, ça tenait. Vos voix sont devenues toutes petites. Les tasses reste dans la paume de Nina. Je reste encore un peu. Une goutte reste collée au bol. L'évier sent encore le cacao.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Sur le tabouret, deux têtes se calment. Victorino, tu l'as vue glisser. Oui, tout près de tes mains. Toi en bas, lui au-dessus, ça tenait. Vos voix sont devenues toutes petites. Les tasses reste dans la paume de Nina. Je reste encore un peu. Une goutte reste collée au bol. L'évier sent encore le cacao.</t>
+          <t>Sur le tabouret, deux têtes se calment. J'ai vu le fond, moi aussi. Oui, tu étais assez haute. Toi en bas, lui au-dessus, ça tenait. Vos voix sont devenues toutes petites. Les tasses reste dans la paume de Nina. Je reste encore un peu. Une goutte reste collée au bol. L'évier sent encore le cacao.</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -13351,8 +13351,8 @@
       <c r="AW69" t="inlineStr">
         <is>
           <t>narrateur|Sur le tabouret, deux têtes se calment.
-enfant-f|Victorino, tu l'as vue glisser.
-copain|Oui, tout près de tes mains.
+enfant-f|J'ai vu le fond, moi aussi.
+copain|Oui, tu étais assez haute.
 papa|Toi en bas, lui au-dessus, ça tenait.
 maman|Vos voix sont devenues toutes petites.
 narrateur|Les tasses reste dans la paume de Nina.
@@ -13385,12 +13385,12 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>On tire un peu. Moi aussi, je tire. Victorino lève un torchon, tout haut. Nina glisse le bol, pendant l'ouverture. Le plateau serre le linge, toc. Il est venu vers vous. On l'a repris. Il fume encore. Vos cheveux sentent le linge chaud.</t>
+          <t>On tire le bol, tout doux. Moi aussi, je tire. Victorino enroule un torchon, tout haut. Nina tire l'autre bout, plus bas. Le plateau glisse avec le linge, toc. Le bol est venu vers vous. On le tient. Il fume encore. Vos cheveux sentent le linge chaud.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>On tire un peu. Moi aussi, je tire. Victorino lève un torchon, tout haut. Nina glisse le bol, pendant l'ouverture. Le plateau serre le linge, toc. Il est venu vers vous. On l'a repris. Il fume encore. Vos cheveux sentent le linge chaud.</t>
+          <t>On tire le bol, tout doux. Moi aussi, je tire. Victorino enroule un torchon, tout haut. Nina tire l'autre bout, plus bas. Le plateau glisse avec le linge, toc. Le bol est venu vers vous. On le tient. Il fume encore. Vos cheveux sentent le linge chaud.</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -13525,13 +13525,13 @@
       <c r="AV70" s="2" t="inlineStr"/>
       <c r="AW70" t="inlineStr">
         <is>
-          <t>enfant-f|On tire un peu.
+          <t>enfant-f|On tire le bol, tout doux.
 copain|Moi aussi, je tire.
-narrateur|Victorino lève un torchon, tout haut.
-narrateur|Nina glisse le bol, pendant l'ouverture.
-narrateur|Le plateau serre le linge, toc.
-papa|Il est venu vers vous.
-copain|On l'a repris.
+narrateur|Victorino enroule un torchon, tout haut.
+narrateur|Nina tire l'autre bout, plus bas.
+narrateur|Le plateau glisse avec le linge, toc.
+papa|Le bol est venu vers vous.
+copain|On le tient.
 enfant-f|Il fume encore.
 maman|Vos cheveux sentent le linge chaud.</t>
         </is>
@@ -13560,12 +13560,12 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Le torchon redescend, tout doux. Il est tombé vers nous. On a tiré, tous les deux. Il n'était plus trop coincé. La poudre froisse encore, dans l'air. Le plateau retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des bols. Le radiateur se tait, au fond.</t>
+          <t>Le torchon redescend, tout doux. Le bol est venu vers nous. On a tiré, tous les deux. Il n'était plus trop haut. La poudre danse encore, dans l'air. Le plateau retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des bols. Le radiateur se tait, au fond.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Le torchon redescend, tout doux. Il est tombé vers nous. On a tiré, tous les deux. Il n'était plus trop coincé. La poudre froisse encore, dans l'air. Le plateau retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des bols. Le radiateur se tait, au fond.</t>
+          <t>Le torchon redescend, tout doux. Le bol est venu vers nous. On a tiré, tous les deux. Il n'était plus trop haut. La poudre danse encore, dans l'air. Le plateau retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des bols. Le radiateur se tait, au fond.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -13701,10 +13701,10 @@
       <c r="AW71" t="inlineStr">
         <is>
           <t>narrateur|Le torchon redescend, tout doux.
-copain|Il est tombé vers nous.
+copain|Le bol est venu vers nous.
 enfant-f|On a tiré, tous les deux.
-maman|Il n'était plus trop coincé.
-papa|La poudre froisse encore, dans l'air.
+maman|Il n'était plus trop haut.
+papa|La poudre danse encore, dans l'air.
 narrateur|Le plateau retombe, tout léger.
 enfant-f|On souffle dessus, tout calme.
 narrateur|Un rayon veille près des bols.
@@ -13735,12 +13735,12 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Le plateau se coince sous le joint. Le lait est à nous, Victorino. Je vois le beurre, tout haut ! La poignée reste trop loin pour Nina. Les tasses n'aident pas, trop basses. Un peu d'air froid lève, puis retombe. Ses bras vont jusqu'à la poignée. Toi tu vois le bac, lui le beurre. On peut jouer avec lui ? Vous trouvez, tous les deux ?</t>
+          <t>Nina tape le plateau contre la porte, toc. Le lait est dedans, Victorino. Je vois déjà le beurre, tout haut ! La poignée reste trop loin pour Nina. Les tasses n'ouvrent rien, trop basses. Un souffle froid lève, puis retombe. Ses bras vont jusqu'à la poignée. Toi tu vois le bac, lui le beurre. On ouvre comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Le plateau se coince sous le joint. Le lait est à nous, Victorino. Je vois le beurre, tout haut ! La poignée reste trop loin pour Nina. Les tasses n'aident pas, trop basses. Un peu d'air froid lève, puis retombe. Ses bras vont jusqu'à la poignée. Toi tu vois le bac, lui le beurre. On peut jouer avec lui ? Vous trouvez, tous les deux ?</t>
+          <t>Nina tape le plateau contre la porte, toc. Le lait est dedans, Victorino. Je vois déjà le beurre, tout haut ! La poignée reste trop loin pour Nina. Les tasses n'ouvrent rien, trop basses. Un souffle froid lève, puis retombe. Ses bras vont jusqu'à la poignée. Toi tu vois le bac, lui le beurre. On ouvre comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -13875,15 +13875,15 @@
       <c r="AV72" s="2" t="inlineStr"/>
       <c r="AW72" t="inlineStr">
         <is>
-          <t>narrateur|Le plateau se coince sous le joint.
-enfant-f|Le lait est à nous, Victorino.
-copain|Je vois le beurre, tout haut !
+          <t>narrateur|Nina tape le plateau contre la porte, toc.
+enfant-f|Le lait est dedans, Victorino.
+copain|Je vois déjà le beurre, tout haut !
 narrateur|La poignée reste trop loin pour Nina.
-narrateur|Les tasses n'aident pas, trop basses.
-narrateur|Un peu d'air froid lève, puis retombe.
+narrateur|Les tasses n'ouvrent rien, trop basses.
+narrateur|Un souffle froid lève, puis retombe.
 maman|Ses bras vont jusqu'à la poignée.
 papa|Toi tu vois le bac, lui le beurre.
-enfant-f|On peut jouer avec lui ?
+enfant-f|On ouvre comment, alors ?
 papa|Vous trouvez, tous les deux ?</t>
         </is>
       </c>
@@ -14107,12 +14107,12 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Je me hausse encore. Je tiens les tasses, d'en bas. Les doigts de Victorino touchent la poignée. Elle bouge ! Le lait penche, puis avance. Victorino pose le plateau contre le joint. Tes doigts allaient assez loin. Nina tenait bien le bas. Il est à nous.</t>
+          <t>Je me hausse encore. Je tiens les tasses, d'en bas. Les doigts de Victorino touchent la poignée. Elle bouge ! La bouteille de lait penche, puis avance. Victorino pose le plateau contre le joint. Tes doigts allaient assez loin. Nina tenait bien le bas. Le lait est à nous.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Je me hausse encore. Je tiens les tasses, d'en bas. Les doigts de Victorino touchent la poignée. Elle bouge ! Le lait penche, puis avance. Victorino pose le plateau contre le joint. Tes doigts allaient assez loin. Nina tenait bien le bas. Il est à nous.</t>
+          <t>Je me hausse encore. Je tiens les tasses, d'en bas. Les doigts de Victorino touchent la poignée. Elle bouge ! La bouteille de lait penche, puis avance. Victorino pose le plateau contre le joint. Tes doigts allaient assez loin. Nina tenait bien le bas. Le lait est à nous.</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -14251,11 +14251,11 @@
 enfant-f|Je tiens les tasses, d'en bas.
 narrateur|Les doigts de Victorino touchent la poignée.
 copain|Elle bouge !
-narrateur|Le lait penche, puis avance.
+narrateur|La bouteille de lait penche, puis avance.
 narrateur|Victorino pose le plateau contre le joint.
 papa|Tes doigts allaient assez loin.
 maman|Nina tenait bien le bas.
-copain|Il est à nous.</t>
+copain|Le lait est à nous.</t>
         </is>
       </c>
     </row>
@@ -14282,12 +14282,12 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Au frigo, le cacao sent le lait. Tu l'as fait pencher pour moi. Tu tenais le bas. Le verre sent encore le matin. Le cacao est à vous, maintenant. Le plateau garde un brin de froid. Nina le verse contre la tasse petite. Un rai traverse la vapeur, tout chaud. Le loquet redevient calme, tout seul.</t>
+          <t>Au frigo, le cacao sent le lait. Tu as ouvert, tout haut. Tu tenais les tasses. Le verre sent encore le matin. Le cacao est à vous, maintenant. Le plateau garde un brin de froid. Nina verse dans la tasse petite. Un rai traverse la vapeur, tout chaud. Le loquet redevient calme, tout seul.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Au frigo, le cacao sent le lait. Tu l'as fait pencher pour moi. Tu tenais le bas. Le verre sent encore le matin. Le cacao est à vous, maintenant. Le plateau garde un brin de froid. Nina le verse contre la tasse petite. Un rai traverse la vapeur, tout chaud. Le loquet redevient calme, tout seul.</t>
+          <t>Au frigo, le cacao sent le lait. Tu as ouvert, tout haut. Tu tenais les tasses. Le verre sent encore le matin. Le cacao est à vous, maintenant. Le plateau garde un brin de froid. Nina verse dans la tasse petite. Un rai traverse la vapeur, tout chaud. Le loquet redevient calme, tout seul.</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -14423,12 +14423,12 @@
       <c r="AW75" t="inlineStr">
         <is>
           <t>narrateur|Au frigo, le cacao sent le lait.
-enfant-f|Tu l'as fait pencher pour moi.
-copain|Tu tenais le bas.
+enfant-f|Tu as ouvert, tout haut.
+copain|Tu tenais les tasses.
 maman|Le verre sent encore le matin.
 papa|Le cacao est à vous, maintenant.
 narrateur|Le plateau garde un brin de froid.
-narrateur|Nina le verse contre la tasse petite.
+narrateur|Nina verse dans la tasse petite.
 narrateur|Un rai traverse la vapeur, tout chaud.
 narrateur|Le loquet redevient calme, tout seul.</t>
         </is>
@@ -14457,12 +14457,12 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>J'ouvre le bac du bas ? Oui, tout doux. Nina pousse le plateau, tout près. Papa tient la porte, tout ferme. Nina tire le bac, Victorino veille. Le lait est là ! Je le sens. Vous avez regardé ensemble. Le bac est resté doux.</t>
+          <t>J'ouvre le bac du bas ? Oui, tout doux. Nina pousse le plateau, tout près. Papa tient la porte, tout ferme. Nina tire le bac, Victorino veille. Le lait est là ! Il est tout froid. Vous avez regardé ensemble. Le bac est resté doux.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>J'ouvre le bac du bas ? Oui, tout doux. Nina pousse le plateau, tout près. Papa tient la porte, tout ferme. Nina tire le bac, Victorino veille. Le lait est là ! Je le sens. Vous avez regardé ensemble. Le bac est resté doux.</t>
+          <t>J'ouvre le bac du bas ? Oui, tout doux. Nina pousse le plateau, tout près. Papa tient la porte, tout ferme. Nina tire le bac, Victorino veille. Le lait est là ! Il est tout froid. Vous avez regardé ensemble. Le bac est resté doux.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -14603,7 +14603,7 @@
 narrateur|Papa tient la porte, tout ferme.
 narrateur|Nina tire le bac, Victorino veille.
 enfant-f|Le lait est là !
-copain|Je le sens.
+copain|Il est tout froid.
 maman|Vous avez regardé ensemble.
 papa|Le bac est resté doux.</t>
         </is>
@@ -14632,12 +14632,12 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Près du bac, deux paires de pieds se touchent. Tu l'as posé, d'en bas. Tes bras l'ont fait descendre. Chacun a fait sa part, à sa hauteur. Le bois du bac sèche déjà. Les tasses pose une ombre au bac. Il fume trop, Nina. C'est pour ça. La porte garde le froid, tout proche.</t>
+          <t>Près du bac, deux paires de pieds se touchent. Tu l'as trouvé, d'en bas. Tes yeux gardaient la porte. Chacun a fait sa part, à sa hauteur. Le bois du bac sèche déjà. Les tasses pose une ombre au bac. Il fume trop, Nina. C'est pour ça. La porte garde le froid, tout proche.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Près du bac, deux paires de pieds se touchent. Tu l'as posé, d'en bas. Tes bras l'ont fait descendre. Chacun a fait sa part, à sa hauteur. Le bois du bac sèche déjà. Les tasses pose une ombre au bac. Il fume trop, Nina. C'est pour ça. La porte garde le froid, tout proche.</t>
+          <t>Près du bac, deux paires de pieds se touchent. Tu l'as trouvé, d'en bas. Tes yeux gardaient la porte. Chacun a fait sa part, à sa hauteur. Le bois du bac sèche déjà. Les tasses pose une ombre au bac. Il fume trop, Nina. C'est pour ça. La porte garde le froid, tout proche.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -14773,8 +14773,8 @@
       <c r="AW77" t="inlineStr">
         <is>
           <t>narrateur|Près du bac, deux paires de pieds se touchent.
-copain|Tu l'as posé, d'en bas.
-enfant-f|Tes bras l'ont fait descendre.
+copain|Tu l'as trouvé, d'en bas.
+enfant-f|Tes yeux gardaient la porte.
 papa|Chacun a fait sa part, à sa hauteur.
 maman|Le bois du bac sèche déjà.
 narrateur|Les tasses pose une ombre au bac.
@@ -14807,12 +14807,12 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Reste en haut, Victorino. Je tends, d'ici. Victorino pousse le plateau, tout près. Victorino fait basculer le loquet, tout doux. Le tabouret prend Nina, puis lui. Je le tiens ! Chacun a fait sa part. Il sent le froid. Vos bras n'avaient pas la même longueur.</t>
+          <t>Reste en haut, Victorino. Je tends, d'ici. Victorino pousse le plateau, tout près. Victorino fait basculer le loquet, tout doux. Le tabouret prend Nina, puis lui. Je tiens la bouteille ! Chacun a fait sa part. Elle sent le froid. Vos bras n'avaient pas la même longueur.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Reste en haut, Victorino. Je tends, d'ici. Victorino pousse le plateau, tout près. Victorino fait basculer le loquet, tout doux. Le tabouret prend Nina, puis lui. Je le tiens ! Chacun a fait sa part. Il sent le froid. Vos bras n'avaient pas la même longueur.</t>
+          <t>Reste en haut, Victorino. Je tends, d'ici. Victorino pousse le plateau, tout près. Victorino fait basculer le loquet, tout doux. Le tabouret prend Nina, puis lui. Je tiens la bouteille ! Chacun a fait sa part. Elle sent le froid. Vos bras n'avaient pas la même longueur.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -14952,9 +14952,9 @@
 narrateur|Victorino pousse le plateau, tout près.
 narrateur|Victorino fait basculer le loquet, tout doux.
 narrateur|Le tabouret prend Nina, puis lui.
-enfant-f|Je le tiens !
+enfant-f|Je tiens la bouteille !
 papa|Chacun a fait sa part.
-copain|Il sent le froid.
+copain|Elle sent le froid.
 maman|Vos bras n'avaient pas la même longueur.</t>
         </is>
       </c>
@@ -14982,12 +14982,12 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Un peu de buée reste au frigo. On a tiré ensemble. Sans trop monter. Le tabouret est resté à sa place. Vos mains sentent encore le lait. Nina pose le plateau au rebord. Tu l'as eu, enfin. Il est à nous. La vapeur tremble un peu, puis s'endort.</t>
+          <t>Un peu de buée reste au frigo. On a ouvert ensemble. Sans trop monter. Le tabouret est resté à sa place. Vos mains sentent encore le lait. Nina pose le plateau au rebord. Tu l'as eu, enfin. Il est à nous. La vapeur tremble un peu, puis s'endort.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Un peu de buée reste au frigo. On a tiré ensemble. Sans trop monter. Le tabouret est resté à sa place. Vos mains sentent encore le lait. Nina pose le plateau au rebord. Tu l'as eu, enfin. Il est à nous. La vapeur tremble un peu, puis s'endort.</t>
+          <t>Un peu de buée reste au frigo. On a ouvert ensemble. Sans trop monter. Le tabouret est resté à sa place. Vos mains sentent encore le lait. Nina pose le plateau au rebord. Tu l'as eu, enfin. Il est à nous. La vapeur tremble un peu, puis s'endort.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -15123,7 +15123,7 @@
       <c r="AW79" t="inlineStr">
         <is>
           <t>narrateur|Un peu de buée reste au frigo.
-enfant-f|On a tiré ensemble.
+enfant-f|On a ouvert ensemble.
 copain|Sans trop monter.
 papa|Le tabouret est resté à sa place.
 maman|Vos mains sentent encore le lait.
@@ -15157,12 +15157,12 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Le plateau bute contre un pied de table. Ici, ça sent le bois, Victorino. Je me glisse, trop large ! Ses épaules butent contre le bois de la table. La porcelaine gratte, puis s'arrête, coincée. Les tasses attend au bord, un peu seul. Il a les épaules trop larges, c'est tout. Toi tu passes, lui pas encore. On joue comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>Nina glisse le plateau sous la table, tout bas. On goûte ici, comme une grotte. J'entre, trop large ! Ses épaules butent contre le bois de la table. Une tasse cliquette, trop près d'une chaise. Les tasses attend au bord, un peu seul. Il a les épaules trop larges, c'est tout. Toi tu passes, lui pas encore. On goûte comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Le plateau bute contre un pied de table. Ici, ça sent le bois, Victorino. Je me glisse, trop large ! Ses épaules butent contre le bois de la table. La porcelaine gratte, puis s'arrête, coincée. Les tasses attend au bord, un peu seul. Il a les épaules trop larges, c'est tout. Toi tu passes, lui pas encore. On joue comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>Nina glisse le plateau sous la table, tout bas. On goûte ici, comme une grotte. J'entre, trop large ! Ses épaules butent contre le bois de la table. Une tasse cliquette, trop près d'une chaise. Les tasses attend au bord, un peu seul. Il a les épaules trop larges, c'est tout. Toi tu passes, lui pas encore. On goûte comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -15297,15 +15297,15 @@
       <c r="AV80" s="2" t="inlineStr"/>
       <c r="AW80" t="inlineStr">
         <is>
-          <t>narrateur|Le plateau bute contre un pied de table.
-enfant-f|Ici, ça sent le bois, Victorino.
-copain|Je me glisse, trop large !
+          <t>narrateur|Nina glisse le plateau sous la table, tout bas.
+enfant-f|On goûte ici, comme une grotte.
+copain|J'entre, trop large !
 narrateur|Ses épaules butent contre le bois de la table.
-narrateur|La porcelaine gratte, puis s'arrête, coincée.
+narrateur|Une tasse cliquette, trop près d'une chaise.
 narrateur|Les tasses attend au bord, un peu seul.
 maman|Il a les épaules trop larges, c'est tout.
 papa|Toi tu passes, lui pas encore.
-copain|On joue comment, alors ?
+copain|On goûte comment, alors ?
 papa|Vous trouvez, tous les deux ?</t>
         </is>
       </c>
@@ -15529,12 +15529,12 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Je passe, Victorino. Nina rampe, tout petite, sous la table. Doucement. Nina pousse le plateau sous le bord. Ses doigts trouvent une cuillère perdue. Je la tiens ! Tes épaules étaient assez petites. Une grotte de lumière s'ouvre, à eux. Regarde, Nina. Elle est à nous.</t>
+          <t>Je passe, toi tu restes. Nina rampe, tout petite, sous la table. Je fouette ici, dehors. Nina pousse le plateau sous le bord. Ses doigts trouvent la petite tasse. Je la tiens ! Tes épaules étaient assez petites. Une grotte de vapeur s'ouvre, à eux. Je te verse, d'ici. Elle est à nous.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Je passe, Victorino. Nina rampe, tout petite, sous la table. Doucement. Nina pousse le plateau sous le bord. Ses doigts trouvent une cuillère perdue. Je la tiens ! Tes épaules étaient assez petites. Une grotte de lumière s'ouvre, à eux. Regarde, Nina. Elle est à nous.</t>
+          <t>Je passe, toi tu restes. Nina rampe, tout petite, sous la table. Je fouette ici, dehors. Nina pousse le plateau sous le bord. Ses doigts trouvent la petite tasse. Je la tiens ! Tes épaules étaient assez petites. Une grotte de vapeur s'ouvre, à eux. Je te verse, d'ici. Elle est à nous.</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -15669,15 +15669,15 @@
       <c r="AV82" s="2" t="inlineStr"/>
       <c r="AW82" t="inlineStr">
         <is>
-          <t>enfant-f|Je passe, Victorino.
+          <t>enfant-f|Je passe, toi tu restes.
 narrateur|Nina rampe, tout petite, sous la table.
-copain|Doucement.
+copain|Je fouette ici, dehors.
 narrateur|Nina pousse le plateau sous le bord.
-narrateur|Ses doigts trouvent une cuillère perdue.
+narrateur|Ses doigts trouvent la petite tasse.
 enfant-f|Je la tiens !
 papa|Tes épaules étaient assez petites.
-narrateur|Une grotte de lumière s'ouvre, à eux.
-copain|Regarde, Nina.
+narrateur|Une grotte de vapeur s'ouvre, à eux.
+copain|Je te verse, d'ici.
 enfant-f|Elle est à nous.</t>
         </is>
       </c>
@@ -15705,12 +15705,12 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Sous la table, la grotte sent le bois. Tu es passée, moi je gardais. Tes épaules l'ont laissé ouvert. Vous l'avez, enfin. La cuillère dort sur le bord, au calme. Le plateau tient encore leurs coudes. On reste un peu, Victorino. Un rai brun s'endort sous le bois. La poussière redevient douce, autour.</t>
+          <t>Sous la table, la grotte sent le bois. Tu es passée, moi je fouettais. Tes épaules l'ont laissé ouvert. Vous l'avez, enfin. La petite tasse dort sur le bord, au calme. Le plateau tient encore leurs coudes. On reste un peu, Victorino. Un rai brun s'endort sous le bois. La miette redevient douce, autour.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Sous la table, la grotte sent le bois. Tu es passée, moi je gardais. Tes épaules l'ont laissé ouvert. Vous l'avez, enfin. La cuillère dort sur le bord, au calme. Le plateau tient encore leurs coudes. On reste un peu, Victorino. Un rai brun s'endort sous le bois. La poussière redevient douce, autour.</t>
+          <t>Sous la table, la grotte sent le bois. Tu es passée, moi je fouettais. Tes épaules l'ont laissé ouvert. Vous l'avez, enfin. La petite tasse dort sur le bord, au calme. Le plateau tient encore leurs coudes. On reste un peu, Victorino. Un rai brun s'endort sous le bois. La miette redevient douce, autour.</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -15846,14 +15846,14 @@
       <c r="AW83" t="inlineStr">
         <is>
           <t>narrateur|Sous la table, la grotte sent le bois.
-copain|Tu es passée, moi je gardais.
+copain|Tu es passée, moi je fouettais.
 enfant-f|Tes épaules l'ont laissé ouvert.
 papa|Vous l'avez, enfin.
-maman|La cuillère dort sur le bord, au calme.
+maman|La petite tasse dort sur le bord, au calme.
 narrateur|Le plateau tient encore leurs coudes.
 enfant-f|On reste un peu, Victorino.
 narrateur|Un rai brun s'endort sous le bois.
-narrateur|La poussière redevient douce, autour.</t>
+narrateur|La miette redevient douce, autour.</t>
         </is>
       </c>
     </row>
@@ -15880,12 +15880,12 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>On écarte un peu. Moi aussi, j'écarte. Victorino tire la chaise, tout haut. Nina se glisse, pendant l'ouverture. Le plateau soulève un coin, toc. Il est venu vers vous. On l'a repris. Il fume encore. Vos cheveux sentent le bois chaud.</t>
+          <t>On écarte la chaise. Moi aussi, j'écarte. Victorino tire la chaise, tout haut. Nina se glisse, pendant l'ouverture. Le plateau avance, toc, vers le jour. La place est venue vers vous. Je rentre, de côté. On y est, tous les deux. Vos cheveux sentent le bois chaud.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>On écarte un peu. Moi aussi, j'écarte. Victorino tire la chaise, tout haut. Nina se glisse, pendant l'ouverture. Le plateau soulève un coin, toc. Il est venu vers vous. On l'a repris. Il fume encore. Vos cheveux sentent le bois chaud.</t>
+          <t>On écarte la chaise. Moi aussi, j'écarte. Victorino tire la chaise, tout haut. Nina se glisse, pendant l'ouverture. Le plateau avance, toc, vers le jour. La place est venue vers vous. Je rentre, de côté. On y est, tous les deux. Vos cheveux sentent le bois chaud.</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -16020,14 +16020,14 @@
       <c r="AV84" s="2" t="inlineStr"/>
       <c r="AW84" t="inlineStr">
         <is>
-          <t>enfant-f|On écarte un peu.
+          <t>enfant-f|On écarte la chaise.
 copain|Moi aussi, j'écarte.
 narrateur|Victorino tire la chaise, tout haut.
 narrateur|Nina se glisse, pendant l'ouverture.
-narrateur|Le plateau soulève un coin, toc.
-papa|Il est venu vers vous.
-copain|On l'a repris.
-enfant-f|Il fume encore.
+narrateur|Le plateau avance, toc, vers le jour.
+papa|La place est venue vers vous.
+copain|Je rentre, de côté.
+enfant-f|On y est, tous les deux.
 maman|Vos cheveux sentent le bois chaud.</t>
         </is>
       </c>
@@ -16055,12 +16055,12 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Le bord de table redescend, tout doux. Il est tombé vers nous. On a écarté, tous les deux. Il n'était plus trop coincé. La poudre froisse encore, dans l'air. Le plateau retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des chaises. Le radiateur se tait, contre le mur.</t>
+          <t>Le bord de table redescend, tout doux. Je suis rentré de côté. On a écarté, tous les deux. Il n'était plus trop coincé. La poudre danse encore, dans l'air. Le plateau retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des chaises. Le radiateur se tait, contre le mur.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Le bord de table redescend, tout doux. Il est tombé vers nous. On a écarté, tous les deux. Il n'était plus trop coincé. La poudre froisse encore, dans l'air. Le plateau retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des chaises. Le radiateur se tait, contre le mur.</t>
+          <t>Le bord de table redescend, tout doux. Je suis rentré de côté. On a écarté, tous les deux. Il n'était plus trop coincé. La poudre danse encore, dans l'air. Le plateau retombe, tout léger. On souffle dessus, tout calme. Un rayon veille près des chaises. Le radiateur se tait, contre le mur.</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -16196,10 +16196,10 @@
       <c r="AW85" t="inlineStr">
         <is>
           <t>narrateur|Le bord de table redescend, tout doux.
-copain|Il est tombé vers nous.
+copain|Je suis rentré de côté.
 enfant-f|On a écarté, tous les deux.
 maman|Il n'était plus trop coincé.
-papa|La poudre froisse encore, dans l'air.
+papa|La poudre danse encore, dans l'air.
 narrateur|Le plateau retombe, tout léger.
 enfant-f|On souffle dessus, tout calme.
 narrateur|Un rayon veille près des chaises.
@@ -16230,12 +16230,12 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Papa, écarte un peu ? Je fais un chemin, tout doux. Une chaise s'ouvre, comme une aile. Nina rentre, Victorino reste dehors. Le plateau devient un nid, contre le bois. On se parle à travers. Oui. Vous y arrivez, tous les deux. Deux voix tiennent le même secret.</t>
+          <t>Papa, écarte un peu ? Je fais un chemin, tout doux. Une chaise s'ouvre, comme une aile. Nina rentre, Victorino reste dehors. Le plateau devient un nid, contre le bois. On trinque à travers ? Oui, petite tasse, grande tasse. Vous y arrivez, tous les deux. Deux voix tiennent le même secret.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Papa, écarte un peu ? Je fais un chemin, tout doux. Une chaise s'ouvre, comme une aile. Nina rentre, Victorino reste dehors. Le plateau devient un nid, contre le bois. On se parle à travers. Oui. Vous y arrivez, tous les deux. Deux voix tiennent le même secret.</t>
+          <t>Papa, écarte un peu ? Je fais un chemin, tout doux. Une chaise s'ouvre, comme une aile. Nina rentre, Victorino reste dehors. Le plateau devient un nid, contre le bois. On trinque à travers ? Oui, petite tasse, grande tasse. Vous y arrivez, tous les deux. Deux voix tiennent le même secret.</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -16375,8 +16375,8 @@
 narrateur|Une chaise s'ouvre, comme une aile.
 narrateur|Nina rentre, Victorino reste dehors.
 narrateur|Le plateau devient un nid, contre le bois.
-copain|On se parle à travers.
-enfant-f|Oui.
+copain|On trinque à travers ?
+enfant-f|Oui, petite tasse, grande tasse.
 maman|Vous y arrivez, tous les deux.
 narrateur|Deux voix tiennent le même secret.</t>
         </is>
@@ -16405,12 +16405,12 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Deux têtes se parlent encore, à travers le bois. On s'est parlé à travers. La table vous a laissé la place. Le secret tient encore, tout chaud. Le plateau garde un brin de lait. Regarde-le, Victorino, il fume. Je le vois, d'ici. Le brun reste au chaud, sous le bois. Une chaise redevient calme, tout seule.</t>
+          <t>Deux tasses se parlent encore, à travers le bois. On a trinqué à travers. La table vous a laissé la place. Le secret tient encore, tout chaud. Le plateau garde un brin de lait. Regarde-le, Victorino, il fume. Je le vois, d'ici. Le brun reste au chaud, sous le bois. Une chaise redevient calme, tout seule.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Deux têtes se parlent encore, à travers le bois. On s'est parlé à travers. La table vous a laissé la place. Le secret tient encore, tout chaud. Le plateau garde un brin de lait. Regarde-le, Victorino, il fume. Je le vois, d'ici. Le brun reste au chaud, sous le bois. Une chaise redevient calme, tout seule.</t>
+          <t>Deux tasses se parlent encore, à travers le bois. On a trinqué à travers. La table vous a laissé la place. Le secret tient encore, tout chaud. Le plateau garde un brin de lait. Regarde-le, Victorino, il fume. Je le vois, d'ici. Le brun reste au chaud, sous le bois. Une chaise redevient calme, tout seule.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -16545,8 +16545,8 @@
       <c r="AV87" s="2" t="inlineStr"/>
       <c r="AW87" t="inlineStr">
         <is>
-          <t>narrateur|Deux têtes se parlent encore, à travers le bois.
-copain|On s'est parlé à travers.
+          <t>narrateur|Deux tasses se parlent encore, à travers le bois.
+copain|On a trinqué à travers.
 papa|La table vous a laissé la place.
 maman|Le secret tient encore, tout chaud.
 narrateur|Le plateau garde un brin de lait.
@@ -16574,7 +16574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16673,6 +16673,13 @@
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): TREE-DIF-042 polish Le cacao de Nina, trop haut sur l'étagère
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-042.xlsx
+++ b/stories/arbres/TREE-DIF-042.xlsx
@@ -1197,17 +1197,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>D'habitude, le bidon de cacao cliquette, dans le placard. Là, le placard reste muet. La casserole, elle, fait tic, sur le feu. Les manteaux mouillés sentent la laine, près de la porte. Nina connaît cette cuisine, presque par cœur. Un détail, là-haut, paraît neuf. Le bidon de cacao penche son capuchon, trop haut. Il n'était pas comme ça. Le capuchon penche, c'est vrai. Tu as vu le lait, Nina ? Il fume, dans la casserole. En ce moment, Nina veut deux tasses, avant la peau du lait. Victorino, on fait du cacao, pour deux ? Victorino arrive, plus grand, sans se presser. J'arrive. Le lait va se couvrir, si on attend. Merci, tu as baissé le feu.</t>
+          <t>D'habitude, le bidon de cacao cliquette, dans le placard. Là, le placard reste muet. La casserole, elle, fait tic, sur le feu. Les manteaux mouillés sentent la laine, près de la porte. Une goutte tombe de la manche, sur le carreau. Ça sent la laine mouillée. Nina connaît cette cuisine, presque par cœur. Un détail, là-haut, paraît neuf. Le bidon de cacao penche son capuchon, trop haut. Il n'était pas comme ça. Le capuchon penche, c'est vrai. Tu as vu le lait, Nina ? Il fume, dans la casserole. En ce moment, Nina veut deux tasses, avant la peau du lait. Victorino, on fait du cacao, pour deux ? Victorino arrive, plus grand, sans se presser. Ses épaules passent au-dessus du plan. J'arrive. Le lait va se couvrir, si on attend. Merci, tu as baissé le feu. Le fouet et les tasses sont prêts, près de l'eau.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;D'habitude, le bidon de cacao cliquette, dans le placard. Là, le placard reste muet. La casserole, elle, fait tic, sur le feu. Les manteaux mouillés sentent la laine, près de la porte. Nina connaît cette cuisine, presque par cœur. Un détail, là-haut, paraît neuf. Le bidon de cacao penche son &lt;emphasis level="moderate"&gt;capuchon&lt;/emphasis&gt;, trop haut. Il n'était pas comme ça. Le capuchon penche, c'est vrai. Tu as vu le lait, Nina ? Il fume, dans la casserole. En ce moment, Nina veut deux tasses, avant la peau du lait. Victorino, on fait du cacao, pour deux ? Victorino arrive, plus grand, sans se presser. J'arrive. Le lait va se couvrir, si on attend. Merci, tu as baissé le feu.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;D'habitude, le bidon de cacao cliquette, dans le placard. Là, le placard reste muet. La casserole, elle, fait tic, sur le feu. Les manteaux mouillés sentent la laine, près de la porte. Une goutte tombe de la manche, sur le carreau. Ça sent la laine mouillée. Nina connaît cette cuisine, presque par cœur. Un détail, là-haut, paraît neuf. Le bidon de cacao penche son &lt;emphasis level="moderate"&gt;capuchon&lt;/emphasis&gt;, trop haut. Il n'était pas comme ça. Le capuchon penche, c'est vrai. Tu as vu le lait, Nina ? Il fume, dans la casserole. En ce moment, Nina veut deux tasses, avant la peau du lait. Victorino, on fait du cacao, pour deux ? Victorino arrive, plus grand, sans se presser. Ses épaules passent au-dessus du plan. J'arrive. Le lait va se couvrir, si on attend. Merci, tu as baissé le feu. Le fouet et les tasses sont prêts, près de l'eau.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>D'habitude, le bidon de cacao cliquette, dans le placard. Là, le placard reste muet. La casserole, elle, fait tic, sur le feu. Les manteaux mouillés sentent la laine, près de la porte. Nina connaît cette cuisine, presque par cœur. Un détail, là-haut, paraît neuf. Le bidon de cacao penche son &lt;emphasis&gt;capuchon&lt;/emphasis&gt;, trop haut. Il n'était pas comme ça. Le capuchon penche, c'est vrai. Tu as vu le lait, Nina ? Il fume, dans la casserole. En ce moment, Nina veut deux tasses, avant la peau du lait. Victorino, on fait du cacao, pour deux ? Victorino arrive, plus grand, sans se presser. J'arrive. Le lait va se couvrir, si on attend. Merci, tu as baissé le feu. [pause]</t>
+          <t>D'habitude, le bidon de cacao cliquette, dans le placard. Là, le placard reste muet. La casserole, elle, fait tic, sur le feu. Les manteaux mouillés sentent la laine, près de la porte. Une goutte tombe de la manche, sur le carreau. Ça sent la laine mouillée. Nina connaît cette cuisine, presque par cœur. Un détail, là-haut, paraît neuf. Le bidon de cacao penche son &lt;emphasis&gt;capuchon&lt;/emphasis&gt;, trop haut. Il n'était pas comme ça. Le capuchon penche, c'est vrai. Tu as vu le lait, Nina ? Il fume, dans la casserole. En ce moment, Nina veut deux tasses, avant la peau du lait. Victorino, on fait du cacao, pour deux ? Victorino arrive, plus grand, sans se presser. Ses épaules passent au-dessus du plan. J'arrive. Le lait va se couvrir, si on attend. Merci, tu as baissé le feu. Le fouet et les tasses sont prêts, près de l'eau. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1345,6 +1345,8 @@
 narrateur|Là, le placard reste muet.
 narrateur|La casserole, elle, fait tic, sur le feu.
 narrateur|Les manteaux mouillés sentent la laine, près de la porte.
+narrateur|Une goutte tombe de la manche, sur le carreau.
+enfant-f|Ça sent la laine mouillée.
 narrateur|Nina connaît cette cuisine, presque par cœur.
 narrateur|Un détail, là-haut, paraît neuf.
 narrateur|Le bidon de cacao penche son capuchon, trop haut.
@@ -1355,9 +1357,11 @@
 narrateur|En ce moment, Nina veut deux tasses, avant la peau du lait.
 enfant-f|Victorino, on fait du cacao, pour deux ?
 narrateur|Victorino arrive, plus grand, sans se presser.
+narrateur|Ses épaules passent au-dessus du plan.
 copain|J'arrive.
 papa|Le lait va se couvrir, si on attend.
-papa|Merci, tu as baissé le feu.</t>
+papa|Merci, tu as baissé le feu.
+maman|Le fouet et les tasses sont prêts, près de l'eau.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1389,17 +1393,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Le bidon, le fouet, et les deux tasses attendent. Tu prends quoi d'abord, Nina ?</t>
+          <t>Le bidon, le fouet, et les deux tasses attendent. Le métal luit, trop loin pour les doigts de Nina. Un clic de tiroir, puis le silence des tasses. Tu prends quoi d'abord, Nina ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le bidon, le fouet, et les deux tasses attendent. Tu prends quoi d'abord, Nina ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le bidon, le fouet, et les deux tasses attendent. Le métal luit, trop loin pour les doigts de Nina. Un clic de tiroir, puis le silence des tasses. Tu prends quoi d'abord, Nina ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le bidon, le fouet, et les deux tasses attendent. Tu prends quoi d'abord, Nina ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Le bidon, le fouet, et les deux tasses attendent. Le métal luit, trop loin pour les doigts de Nina. Un clic de tiroir, puis le silence des tasses. Tu prends quoi d'abord, Nina ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -1558,6 +1562,8 @@
       <c r="AW3" t="inlineStr">
         <is>
           <t>narrateur|Le bidon, le fouet, et les deux tasses attendent.
+narrateur|Le métal luit, trop loin pour les doigts de Nina.
+narrateur|Un clic de tiroir, puis le silence des tasses.
 maman|Tu prends quoi d'abord, Nina ?</t>
         </is>
       </c>
@@ -1962,17 +1968,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Contre la hanche. Oui. Il est froid. Il va chauffer dans le lait. Victorino a les genoux plus hauts que Nina. Ses mains touchent le bord du plan. On reste dans la cuisine ? Oui, papa. Le capuchon penche, contre la robe.</t>
+          <t>Contre la hanche. Oui. Il est froid. Il va chauffer dans le lait. Victorino a les genoux plus hauts que Nina. Ses mains touchent le bord du plan. On reste dans la cuisine ? Oui, papa. Le capuchon penche, contre la robe. Un peu de poudre reste au creux de sa paume. Vous emportez aussi le fouet, et les tasses.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Contre la hanche. Oui. Il est froid. Il va chauffer dans le lait. Victorino a les genoux plus hauts que Nina. Ses mains touchent le bord du plan. On reste dans la cuisine ? Oui, papa. Le capuchon penche, contre la robe.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Contre la hanche. Oui. Il est froid. Il va chauffer dans le lait. Victorino a les genoux plus hauts que Nina. Ses mains touchent le bord du plan. On reste dans la cuisine ? Oui, papa. Le capuchon penche, contre la robe. Un peu de poudre reste au creux de sa paume. Vous emportez aussi le fouet, et les tasses.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Contre la hanche. Oui. Il est froid. Il va chauffer dans le lait. Victorino a les genoux plus hauts que Nina. Ses mains touchent le bord du plan. On reste dans la cuisine ? Oui, papa. Le capuchon penche, contre la robe. [pause]</t>
+          <t>Contre la hanche. Oui. Il est froid. Il va chauffer dans le lait. Victorino a les genoux plus hauts que Nina. Ses mains touchent le bord du plan. On reste dans la cuisine ? Oui, papa. Le capuchon penche, contre la robe. Un peu de poudre reste au creux de sa paume. Vous emportez aussi le fouet, et les tasses. [pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2114,7 +2120,9 @@
 narrateur|Ses mains touchent le bord du plan.
 papa|On reste dans la cuisine ?
 enfant-f|Oui, papa.
-narrateur|Le capuchon penche, contre la robe.</t>
+narrateur|Le capuchon penche, contre la robe.
+narrateur|Un peu de poudre reste au creux de sa paume.
+maman|Vous emportez aussi le fouet, et les tasses.</t>
         </is>
       </c>
     </row>
@@ -2141,17 +2149,17 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Le bidon tape la hanche, froid. L'étagère reste trop haute. Le frigo garde son lait, trop loin. Sous la table, l'ombre est basse. Nina, vous mélangez où ?</t>
+          <t>Le bidon tape la hanche, froid. L'étagère reste trop haute. Le frigo garde son lait, trop loin. Sous la table, l'ombre est basse. Le capuchon penche, à chaque pas. Nina, vous mélangez où ?</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le bidon tape la hanche, froid. L'étagère reste trop haute. Le frigo garde son lait, trop loin. Sous la table, l'ombre est basse. Nina, vous mélangez où ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le bidon tape la hanche, froid. L'étagère reste trop haute. Le frigo garde son lait, trop loin. Sous la table, l'ombre est basse. Le capuchon penche, à chaque pas. Nina, vous mélangez où ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le bidon tape la hanche, froid. L'étagère reste trop haute. Le frigo garde son lait, trop loin. Sous la table, l'ombre est basse. Nina, vous mélangez où ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Le bidon tape la hanche, froid. L'étagère reste trop haute. Le frigo garde son lait, trop loin. Sous la table, l'ombre est basse. Le capuchon penche, à chaque pas. Nina, vous mélangez où ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -2313,6 +2321,7 @@
 narrateur|L'étagère reste trop haute.
 narrateur|Le frigo garde son lait, trop loin.
 narrateur|Sous la table, l'ombre est basse.
+narrateur|Le capuchon penche, à chaque pas.
 papa|Nina, vous mélangez où ?</t>
         </is>
       </c>
@@ -2533,17 +2542,17 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>L'étagère attend, trop haute. Les bras, le tabouret, ou le torchon ensemble ?</t>
+          <t>L'étagère attend, trop haute. Nina pose une main sur le bois, sans sauter. Les bras, le tabouret, ou le torchon ensemble ?</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;L'étagère attend, trop haute. Les bras, le tabouret, ou le torchon ensemble ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;L'étagère attend, trop haute. Nina pose une main sur le bois, sans sauter. Les bras, le tabouret, ou le torchon ensemble ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;L'étagère attend, trop haute. Les bras, le tabouret, ou le torchon ensemble ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;L'étagère attend, trop haute. Nina pose une main sur le bois, sans sauter. Les bras, le tabouret, ou le torchon ensemble ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -2702,6 +2711,7 @@
       <c r="AW9" t="inlineStr">
         <is>
           <t>narrateur|L'étagère attend, trop haute.
+narrateur|Nina pose une main sur le bois, sans sauter.
 papa|Les bras, le tabouret, ou le torchon ensemble ?</t>
         </is>
       </c>
@@ -4046,17 +4056,17 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>La poignée attend, trop loin. La poignée, le bac, ou le tabouret ?</t>
+          <t>La poignée attend, trop loin. Nina pose une main sur le joint, sans tirer. La poignée, le bac, ou le tabouret ?</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;La poignée attend, trop loin. La poignée, le bac, ou le tabouret ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;La poignée attend, trop loin. Nina pose une main sur le joint, sans tirer. La poignée, le bac, ou le tabouret ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;La poignée attend, trop loin. La poignée, le bac, ou le tabouret ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;La poignée attend, trop loin. Nina pose une main sur le joint, sans tirer. La poignée, le bac, ou le tabouret ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
@@ -4215,6 +4225,7 @@
       <c r="AW17" t="inlineStr">
         <is>
           <t>narrateur|La poignée attend, trop loin.
+narrateur|Nina pose une main sur le joint, sans tirer.
 maman|La poignée, le bac, ou le tabouret ?</t>
         </is>
       </c>
@@ -5559,17 +5570,17 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>L'ombre sous la table attend. Le passage, écarter, ou un dessous un dessus ?</t>
+          <t>L'ombre sous la table attend. Nina pose une main sur le pied, sans forcer. Le passage, écarter, ou un dessous un dessus ?</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;L'ombre sous la table attend. Le passage, écarter, ou un dessous un dessus ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;L'ombre sous la table attend. Nina pose une main sur le pied, sans forcer. Le passage, écarter, ou un dessous un dessus ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;L'ombre sous la table attend. Le passage, écarter, ou un dessous un dessus ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;L'ombre sous la table attend. Nina pose une main sur le pied, sans forcer. Le passage, écarter, ou un dessous un dessus ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
@@ -5728,6 +5739,7 @@
       <c r="AW25" t="inlineStr">
         <is>
           <t>narrateur|L'ombre sous la table attend.
+narrateur|Nina pose une main sur le pied, sans forcer.
 papa|Le passage, écarter, ou un dessous un dessus ?</t>
         </is>
       </c>
@@ -7257,17 +7269,17 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Dans la poche. Oui. J'entends le clic. Ne le sors pas. Victorino se baisse, trop long, trop vite. Une mèche saute au-dessus du pichet. Vos mains, au-dessus du plateau ? Oui, maman. Le capuchon penche, près du fouet.</t>
+          <t>Dans la poche. Oui. J'entends le clic. Ne le sors pas. Victorino se baisse, trop long, trop vite. Une mèche saute au-dessus du pichet. Vos mains, au-dessus du plateau ? Oui, maman. Le capuchon penche, près du fouet. Le clic dans la poche rythme ses pas. Le bidon et les tasses voyagent avec vous.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Dans la poche. Oui. J'entends le clic. Ne le sors pas. Victorino se baisse, trop long, trop vite. Une mèche saute au-dessus du pichet. Vos mains, au-dessus du plateau ? Oui, maman. Le capuchon penche, près du fouet.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Dans la poche. Oui. J'entends le clic. Ne le sors pas. Victorino se baisse, trop long, trop vite. Une mèche saute au-dessus du pichet. Vos mains, au-dessus du plateau ? Oui, maman. Le capuchon penche, près du fouet. Le clic dans la poche rythme ses pas. Le bidon et les tasses voyagent avec vous.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Dans la poche. Oui. J'entends le clic. Ne le sors pas. Victorino se baisse, trop long, trop vite. Une mèche saute au-dessus du pichet. Vos mains, au-dessus du plateau ? Oui, maman. Le capuchon penche, près du fouet. [pause]</t>
+          <t>Dans la poche. Oui. J'entends le clic. Ne le sors pas. Victorino se baisse, trop long, trop vite. Une mèche saute au-dessus du pichet. Vos mains, au-dessus du plateau ? Oui, maman. Le capuchon penche, près du fouet. Le clic dans la poche rythme ses pas. Le bidon et les tasses voyagent avec vous. [pause]</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -7409,7 +7421,9 @@
 narrateur|Une mèche saute au-dessus du pichet.
 maman|Vos mains, au-dessus du plateau ?
 copain|Oui, maman.
-narrateur|Le capuchon penche, près du fouet.</t>
+narrateur|Le capuchon penche, près du fouet.
+narrateur|Le clic dans la poche rythme ses pas.
+papa|Le bidon et les tasses voyagent avec vous.</t>
         </is>
       </c>
     </row>
@@ -7436,17 +7450,17 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Le fouet frotte la poche, un peu rêche. L'étagère, le frigo, ou sous la table. Vous mélangez où, Nina ?</t>
+          <t>Le fouet frotte la poche, un peu rêche. L'étagère, le frigo, ou sous la table. Le capuchon penche, à chaque pas. Vous mélangez où, Nina ?</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le fouet frotte la poche, un peu rêche. L'étagère, le frigo, ou sous la table. Vous mélangez où, Nina ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le fouet frotte la poche, un peu rêche. L'étagère, le frigo, ou sous la table. Le capuchon penche, à chaque pas. Vous mélangez où, Nina ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le fouet frotte la poche, un peu rêche. L'étagère, le frigo, ou sous la table. Vous mélangez où, Nina ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Le fouet frotte la poche, un peu rêche. L'étagère, le frigo, ou sous la table. Le capuchon penche, à chaque pas. Vous mélangez où, Nina ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
@@ -7606,6 +7620,7 @@
         <is>
           <t>narrateur|Le fouet frotte la poche, un peu rêche.
 narrateur|L'étagère, le frigo, ou sous la table.
+narrateur|Le capuchon penche, à chaque pas.
 maman|Vous mélangez où, Nina ?</t>
         </is>
       </c>
@@ -7825,17 +7840,17 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>L'étagère attend, trop haute. Les bras, le tabouret, ou le torchon ensemble ?</t>
+          <t>L'étagère attend, trop haute. Nina pose une main sur le bois, sans sauter. Les bras, le tabouret, ou le torchon ensemble ?</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;L'étagère attend, trop haute. Les bras, le tabouret, ou le torchon ensemble ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;L'étagère attend, trop haute. Nina pose une main sur le bois, sans sauter. Les bras, le tabouret, ou le torchon ensemble ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;L'étagère attend, trop haute. Les bras, le tabouret, ou le torchon ensemble ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;L'étagère attend, trop haute. Nina pose une main sur le bois, sans sauter. Les bras, le tabouret, ou le torchon ensemble ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
@@ -7994,6 +8009,7 @@
       <c r="AW37" t="inlineStr">
         <is>
           <t>narrateur|L'étagère attend, trop haute.
+narrateur|Nina pose une main sur le bois, sans sauter.
 papa|Les bras, le tabouret, ou le torchon ensemble ?</t>
         </is>
       </c>
@@ -9337,17 +9353,17 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>La poignée attend, trop loin. La poignée, le bac, ou le tabouret ?</t>
+          <t>La poignée attend, trop loin. Nina pose une main sur le joint, sans tirer. La poignée, le bac, ou le tabouret ?</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;La poignée attend, trop loin. La poignée, le bac, ou le tabouret ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;La poignée attend, trop loin. Nina pose une main sur le joint, sans tirer. La poignée, le bac, ou le tabouret ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;La poignée attend, trop loin. La poignée, le bac, ou le tabouret ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;La poignée attend, trop loin. Nina pose une main sur le joint, sans tirer. La poignée, le bac, ou le tabouret ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr"/>
@@ -9506,6 +9522,7 @@
       <c r="AW45" t="inlineStr">
         <is>
           <t>narrateur|La poignée attend, trop loin.
+narrateur|Nina pose une main sur le joint, sans tirer.
 maman|La poignée, le bac, ou le tabouret ?</t>
         </is>
       </c>
@@ -10850,17 +10867,17 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>L'ombre sous la table attend. Le passage, écarter, ou un dessous un dessus ?</t>
+          <t>L'ombre sous la table attend. Nina pose une main sur le pied, sans forcer. Le passage, écarter, ou un dessous un dessus ?</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;L'ombre sous la table attend. Le passage, écarter, ou un dessous un dessus ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;L'ombre sous la table attend. Nina pose une main sur le pied, sans forcer. Le passage, écarter, ou un dessous un dessus ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;L'ombre sous la table attend. Le passage, écarter, ou un dessous un dessus ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;L'ombre sous la table attend. Nina pose une main sur le pied, sans forcer. Le passage, écarter, ou un dessous un dessus ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr"/>
@@ -11019,6 +11036,7 @@
       <c r="AW53" t="inlineStr">
         <is>
           <t>narrateur|L'ombre sous la table attend.
+narrateur|Nina pose une main sur le pied, sans forcer.
 papa|Le passage, écarter, ou un dessous un dessus ?</t>
         </is>
       </c>
@@ -12548,17 +12566,17 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Sur le plateau. Oui. La grande est à moi ? Oui, la petite est à moi. Le pull de Victorino laisse ses poignets nus. Nina, plus courte, tient le plateau des deux mains. On y va, tous les quatre ? Oui. Le capuchon penche, au-dessus des tasses.</t>
+          <t>Sur le plateau. Oui. La grande est à moi ? Oui, la petite est à moi. Le pull de Victorino laisse ses poignets nus. Nina, plus courte, tient le plateau des deux mains. On y va, tous les quatre ? Oui. Le capuchon penche, au-dessus des tasses. La petite tasse tremble, puis se tient. Le bidon et le fouet partent avec le plateau.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sur le plateau. Oui. La grande est à moi ? Oui, la petite est à moi. Le pull de Victorino laisse ses poignets nus. Nina, plus courte, tient le plateau des deux mains. On y va, tous les quatre ? Oui. Le capuchon penche, au-dessus des tasses.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sur le plateau. Oui. La grande est à moi ? Oui, la petite est à moi. Le pull de Victorino laisse ses poignets nus. Nina, plus courte, tient le plateau des deux mains. On y va, tous les quatre ? Oui. Le capuchon penche, au-dessus des tasses. La petite tasse tremble, puis se tient. Le bidon et le fouet partent avec le plateau.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Sur le plateau. Oui. La grande est à moi ? Oui, la petite est à moi. Le pull de Victorino laisse ses poignets nus. Nina, plus courte, tient le plateau des deux mains. On y va, tous les quatre ? Oui. Le capuchon penche, au-dessus des tasses. [pause]</t>
+          <t>Sur le plateau. Oui. La grande est à moi ? Oui, la petite est à moi. Le pull de Victorino laisse ses poignets nus. Nina, plus courte, tient le plateau des deux mains. On y va, tous les quatre ? Oui. Le capuchon penche, au-dessus des tasses. La petite tasse tremble, puis se tient. Le bidon et le fouet partent avec le plateau. [pause]</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr"/>
@@ -12700,7 +12718,9 @@
 narrateur|Nina, plus courte, tient le plateau des deux mains.
 papa|On y va, tous les quatre ?
 enfant-f|Oui.
-narrateur|Le capuchon penche, au-dessus des tasses.</t>
+narrateur|Le capuchon penche, au-dessus des tasses.
+narrateur|La petite tasse tremble, puis se tient.
+maman|Le bidon et le fouet partent avec le plateau.</t>
         </is>
       </c>
     </row>
@@ -12727,17 +12747,17 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Les tasses s'entrechoquent, sur le plateau. L'étagère, le frigo, ou sous la table. Vous mélangez où, Nina ?</t>
+          <t>Les tasses s'entrechoquent, sur le plateau. L'étagère, le frigo, ou sous la table. Le capuchon penche, à chaque pas. Vous mélangez où, Nina ?</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Les tasses s'entrechoquent, sur le plateau. L'étagère, le frigo, ou sous la table. Vous mélangez où, Nina ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Les tasses s'entrechoquent, sur le plateau. L'étagère, le frigo, ou sous la table. Le capuchon penche, à chaque pas. Vous mélangez où, Nina ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Les tasses s'entrechoquent, sur le plateau. L'étagère, le frigo, ou sous la table. Vous mélangez où, Nina ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Les tasses s'entrechoquent, sur le plateau. L'étagère, le frigo, ou sous la table. Le capuchon penche, à chaque pas. Vous mélangez où, Nina ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr"/>
@@ -12897,6 +12917,7 @@
         <is>
           <t>narrateur|Les tasses s'entrechoquent, sur le plateau.
 narrateur|L'étagère, le frigo, ou sous la table.
+narrateur|Le capuchon penche, à chaque pas.
 papa|Vous mélangez où, Nina ?</t>
         </is>
       </c>
@@ -13116,17 +13137,17 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>L'étagère attend, trop haute. Les bras, le tabouret, ou le torchon ensemble ?</t>
+          <t>L'étagère attend, trop haute. Nina pose une main sur le bois, sans sauter. Les bras, le tabouret, ou le torchon ensemble ?</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;L'étagère attend, trop haute. Les bras, le tabouret, ou le torchon ensemble ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;L'étagère attend, trop haute. Nina pose une main sur le bois, sans sauter. Les bras, le tabouret, ou le torchon ensemble ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;L'étagère attend, trop haute. Les bras, le tabouret, ou le torchon ensemble ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;L'étagère attend, trop haute. Nina pose une main sur le bois, sans sauter. Les bras, le tabouret, ou le torchon ensemble ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr"/>
@@ -13285,6 +13306,7 @@
       <c r="AW65" t="inlineStr">
         <is>
           <t>narrateur|L'étagère attend, trop haute.
+narrateur|Nina pose une main sur le bois, sans sauter.
 papa|Les bras, le tabouret, ou le torchon ensemble ?</t>
         </is>
       </c>
@@ -14628,17 +14650,17 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>La poignée attend, trop loin. La poignée, le bac, ou le tabouret ?</t>
+          <t>La poignée attend, trop loin. Nina pose une main sur le joint, sans tirer. La poignée, le bac, ou le tabouret ?</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;La poignée attend, trop loin. La poignée, le bac, ou le tabouret ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;La poignée attend, trop loin. Nina pose une main sur le joint, sans tirer. La poignée, le bac, ou le tabouret ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;La poignée attend, trop loin. La poignée, le bac, ou le tabouret ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;La poignée attend, trop loin. Nina pose une main sur le joint, sans tirer. La poignée, le bac, ou le tabouret ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr"/>
@@ -14797,6 +14819,7 @@
       <c r="AW73" t="inlineStr">
         <is>
           <t>narrateur|La poignée attend, trop loin.
+narrateur|Nina pose une main sur le joint, sans tirer.
 maman|La poignée, le bac, ou le tabouret ?</t>
         </is>
       </c>
@@ -16140,17 +16163,17 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>L'ombre sous la table attend. Le passage, écarter, ou un dessous un dessus ?</t>
+          <t>L'ombre sous la table attend. Nina pose une main sur le pied, sans forcer. Le passage, écarter, ou un dessous un dessus ?</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;L'ombre sous la table attend. Le passage, écarter, ou un dessous un dessus ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;L'ombre sous la table attend. Nina pose une main sur le pied, sans forcer. Le passage, écarter, ou un dessous un dessus ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;L'ombre sous la table attend. Le passage, écarter, ou un dessous un dessus ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;L'ombre sous la table attend. Nina pose une main sur le pied, sans forcer. Le passage, écarter, ou un dessous un dessus ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr"/>
@@ -16309,6 +16332,7 @@
       <c r="AW81" t="inlineStr">
         <is>
           <t>narrateur|L'ombre sous la table attend.
+narrateur|Nina pose une main sur le pied, sans forcer.
 papa|Le passage, écarter, ou un dessous un dessus ?</t>
         </is>
       </c>
@@ -17455,7 +17479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17568,6 +17592,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>